<commit_message>
Corregir datación relativa en F-021
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pascual\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CB6C5A2-3771-40DB-9B9E-99D433440991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E43160-D5B5-40FC-BDBA-0C4BA5C9F266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="225">
   <si>
     <t>Periodo</t>
   </si>
@@ -1077,9 +1077,6 @@
   </si>
   <si>
     <t>Crossognathiformes</t>
-  </si>
-  <si>
-    <t>108 -113 millones de años</t>
   </si>
   <si>
     <t>Cuenca de Araripe</t>
@@ -2703,10 +2700,10 @@
         <v>106</v>
       </c>
       <c r="F22" t="s">
+        <v>205</v>
+      </c>
+      <c r="G22" t="s">
         <v>220</v>
-      </c>
-      <c r="G22" t="s">
-        <v>221</v>
       </c>
       <c r="H22" t="s">
         <v>34</v>
@@ -2750,19 +2747,19 @@
         <v>127</v>
       </c>
       <c r="C23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
       <c r="E23" t="s">
+        <v>221</v>
+      </c>
+      <c r="F23" t="s">
         <v>222</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>223</v>
-      </c>
-      <c r="G23" t="s">
-        <v>224</v>
       </c>
       <c r="H23" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Confirmar correcciones paleontológicas en F-013, F-015, F-016 y F-017
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pascual\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E43160-D5B5-40FC-BDBA-0C4BA5C9F266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3B1FCC-3B12-40F2-9B40-10B026081864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,9 +612,6 @@
     <t>Ejemplar pulido de cefalópodo nautiloideo de concha recta, conservado en sección longitudinal ligeramente oblicua. Se distingue con claridad el fragmocono, con cámaras internas separadas por septos curvos, rellenos de calcita clara, que contrastan con la matriz caliza oscura.</t>
   </si>
   <si>
-    <t>Ejemplar de ammonite planiespiral, con enrollamiento evoluto y ombligo amplio, característico del género Perisphinctes. La concha presenta costulación radial fuerte y densa, con costillas simples que se bifurcan hacia el borde externo, un rasgo diagnóstico del grupo. El relieve costal se conserva bien, aunque con desgaste parcial en algunos sectores. Se observan variaciones cromáticas naturales (grises, ocres y rojizos) debidas a procesos de diagénesis ferruginosa en la matriz calcárea. El área ventral aparece redondeada, sin quilla marcada. El tamaño y robustez sugieren un ejemplar adulto o subadulto.</t>
-  </si>
-  <si>
     <t>Ammonite</t>
   </si>
   <si>
@@ -624,19 +621,310 @@
     <t>Cuenca del Volga (probable)</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada, característica del género </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
+    <t>Cretácico superior</t>
+  </si>
+  <si>
+    <t>Cretácico inferior</t>
+  </si>
+  <si>
+    <t>Helecho arborescente</t>
+  </si>
+  <si>
+    <t>Carbonífero superior</t>
+  </si>
+  <si>
+    <t>Impresión fósil de fronde de helecho con pinnas bien definidas y pínnulos paralelos, conservada en lutita oscura. Procede de depósitos pantanosos del Carbonífero, asociados a ambientes de bosque tropical húmedo y formaciones carboníferas.</t>
+  </si>
+  <si>
+    <t>Gastropoda</t>
+  </si>
+  <si>
+    <t>Caenogastropoda</t>
+  </si>
+  <si>
+    <t>Turritella sp.</t>
+  </si>
+  <si>
+    <t>Turritella</t>
+  </si>
+  <si>
+    <t>Concha fósil de gasterópodo marino de morfología turriculada, formada por numerosas vueltas helicoidales estrechas y regulares. Ejemplar conservado parcialmente en matriz calcarenítica, típico de ambientes marinos someros del Neógeno (Mioceno), muy comunes en el Algarve portugués.</t>
+  </si>
+  <si>
+    <t>Neógeno</t>
+  </si>
+  <si>
+    <t>Mioceno</t>
+  </si>
+  <si>
+    <t>Parcialmente conservado</t>
+  </si>
+  <si>
+    <t>Gymnospermae</t>
+  </si>
+  <si>
+    <t>Xilópalo</t>
+  </si>
+  <si>
+    <t>Corte transversal de tronco silicificado con preservación detallada del tejido vascular y anillos de crecimiento, testimonio de antiguos bosques mesozoicos del Gondwana.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corte transversal </t>
+  </si>
+  <si>
+    <t>Coniferophytina</t>
+  </si>
+  <si>
+    <t>Araucariales</t>
+  </si>
+  <si>
+    <t>Ejemplar conservado como impresión en caliza, correspondiente a un pez óseo de cuerpo fusiforme, típico de ambientes marinos someros del Cretácico temprano.</t>
+  </si>
+  <si>
+    <t>Pez fósil</t>
+  </si>
+  <si>
+    <t>Diente de tiburón fósil</t>
+  </si>
+  <si>
+    <t>Diente perteneciente a un gran tiburón lamniforme primitivo, antecesor del linaje que culminará en Otodus megalodon. Ejemplar conservado en matriz marina.</t>
+  </si>
+  <si>
+    <t>Trilobite enrollado en posición defensiva, ojos grandes y claramente visibles, con lentes individuales (ojo esquizocroal), cefalón robusto, bien mineralizado, tórax con segmentos marcados y regulares, pigidio relativamente pequeño, exoesqueleto oscuro, calcítico, matriz carbonatada compacta típica del Anti-Atlas.</t>
+  </si>
+  <si>
+    <t>Dimensiones</t>
+  </si>
+  <si>
+    <t>657 gr</t>
+  </si>
+  <si>
+    <t>290 gr</t>
+  </si>
+  <si>
+    <t>30 gr</t>
+  </si>
+  <si>
+    <t>311 gr</t>
+  </si>
+  <si>
+    <t>42 gr</t>
+  </si>
+  <si>
+    <t>516 gr</t>
+  </si>
+  <si>
+    <t>313 gr</t>
+  </si>
+  <si>
+    <t>1,7 Kg</t>
+  </si>
+  <si>
+    <t>2,4 Kg</t>
+  </si>
+  <si>
+    <t>7x10 cm</t>
+  </si>
+  <si>
+    <t>8x8 cm</t>
+  </si>
+  <si>
+    <t>2x5 cm</t>
+  </si>
+  <si>
+    <t>7x9 cm</t>
+  </si>
+  <si>
+    <t>17x25 cm</t>
+  </si>
+  <si>
+    <t>2x6 cm</t>
+  </si>
+  <si>
+    <t>10x18 cm</t>
+  </si>
+  <si>
+    <t>7x13 cm</t>
+  </si>
+  <si>
+    <t>21x14 cm</t>
+  </si>
+  <si>
+    <t>36 gr</t>
+  </si>
+  <si>
+    <t>4x6 cm</t>
+  </si>
+  <si>
+    <t>20 gr</t>
+  </si>
+  <si>
+    <t>2x8</t>
+  </si>
+  <si>
+    <t>Pulido industrial- Cianocrilato</t>
+  </si>
+  <si>
+    <t>87 gr</t>
+  </si>
+  <si>
+    <t>5,5x6,5 cm</t>
+  </si>
+  <si>
+    <t>6,8 × 7 cm</t>
+  </si>
+  <si>
+    <t>Hammatoceras Subinsigne</t>
+  </si>
+  <si>
+    <t>900 gr</t>
+  </si>
+  <si>
+    <t>15x12 cm</t>
+  </si>
+  <si>
+    <t>Mantelliceras sp.</t>
+  </si>
+  <si>
+    <t>2,350 Kg</t>
+  </si>
+  <si>
+    <t>15x18 cm</t>
+  </si>
+  <si>
+    <t>1,5 Kg</t>
+  </si>
+  <si>
+    <t>16x20 cm</t>
+  </si>
+  <si>
+    <t>150 gr</t>
+  </si>
+  <si>
+    <t>10,5x12 cm</t>
+  </si>
+  <si>
+    <t>78 gr</t>
+  </si>
+  <si>
+    <t>605 gr</t>
+  </si>
+  <si>
+    <t>8x5,7 cm</t>
+  </si>
+  <si>
+    <t>12x14 cm</t>
+  </si>
+  <si>
+    <t>270 gr</t>
+  </si>
+  <si>
+    <t>89 gr</t>
+  </si>
+  <si>
+    <t>4,7x10,7 cm</t>
+  </si>
+  <si>
+    <t>8,3x5,2 cm</t>
+  </si>
+  <si>
+    <t>Acadoparadoxides sp.</t>
+  </si>
+  <si>
+    <t>Zona de Zagora (probable)</t>
+  </si>
+  <si>
+    <t>Jurásico superior</t>
+  </si>
+  <si>
+    <t>445 - 460 millones de años</t>
+  </si>
+  <si>
+    <t>Flexicalymene Ouzregui sp.</t>
+  </si>
+  <si>
+    <t>485–500 millones de años</t>
+  </si>
+  <si>
+    <t>Corynexochida</t>
+  </si>
+  <si>
+    <t>Illaenus sp.</t>
+  </si>
+  <si>
+    <t>Yacimientos del río Volkhov (probable)</t>
+  </si>
+  <si>
+    <t>445 - 450 millones de años</t>
+  </si>
+  <si>
+    <t>Género</t>
+  </si>
+  <si>
+    <t>Phacops sp.</t>
+  </si>
+  <si>
+    <t>Región de Alnif</t>
+  </si>
+  <si>
+    <t>Orthoceras sp.</t>
+  </si>
+  <si>
+    <t>360 - 410 millones de años</t>
+  </si>
+  <si>
+    <t>360 - 390 millones de años</t>
+  </si>
+  <si>
+    <t>Región de Erfoud</t>
+  </si>
+  <si>
+    <t>Formaciones de caliza negra del Sahara</t>
+  </si>
+  <si>
+    <t>Jurásico medio</t>
+  </si>
+  <si>
+    <t>Cámbrico medio</t>
+  </si>
+  <si>
+    <t>Ordovícico superior</t>
+  </si>
+  <si>
+    <t>Ordovícico medio</t>
+  </si>
+  <si>
+    <t>Ordovícico tardío</t>
+  </si>
+  <si>
+    <t>Devónico superior</t>
+  </si>
+  <si>
+    <t>460 – 470 millones de años</t>
+  </si>
+  <si>
+    <t>170 - 174 millones de años</t>
+  </si>
+  <si>
+    <t>163 - 166 millones de años</t>
+  </si>
+  <si>
+    <t>94 - 100 millones de años</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Región de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Perisphinctes</t>
+      <t>Agadir</t>
     </r>
     <r>
       <rPr>
@@ -646,309 +934,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Jurásico medio y constituye un importante fósil guía para este intervalo.</t>
-    </r>
-  </si>
-  <si>
-    <t>Cretácico superior</t>
-  </si>
-  <si>
-    <t>Ammonite de concha planiespiral evoluta, caracterizada por costillas gruesas y regulares que alcanzan el margen externo, donde forman un contorno dentado. Pertenece al género Acanthoceras, un grupo típico del Cretácico superior, ampliamente utilizado como fósil guía del Cenomaniense. Conservado en matriz calcárea con alteraciones ferruginosas, procedente de depósitos marinos someros del norte de África.</t>
-  </si>
-  <si>
-    <t>Cretácico inferior</t>
-  </si>
-  <si>
-    <t>Ammonite del Cretácico inferior con concha planiespiral evoluta. El pulido revela la compleja red de suturas internas, correspondientes a los tabiques que separaban las cámaras de flotación. Estas estructuras permitían al animal regular su posición en la columna de agua. Ejemplar procedente de depósitos marinos del Anti-Atlas marroquí.</t>
-  </si>
-  <si>
-    <t>Helecho arborescente</t>
-  </si>
-  <si>
-    <t>Carbonífero superior</t>
-  </si>
-  <si>
-    <t>Impresión fósil de fronde de helecho con pinnas bien definidas y pínnulos paralelos, conservada en lutita oscura. Procede de depósitos pantanosos del Carbonífero, asociados a ambientes de bosque tropical húmedo y formaciones carboníferas.</t>
-  </si>
-  <si>
-    <t>Gastropoda</t>
-  </si>
-  <si>
-    <t>Caenogastropoda</t>
-  </si>
-  <si>
-    <t>Turritella sp.</t>
-  </si>
-  <si>
-    <t>Turritella</t>
-  </si>
-  <si>
-    <t>Concha fósil de gasterópodo marino de morfología turriculada, formada por numerosas vueltas helicoidales estrechas y regulares. Ejemplar conservado parcialmente en matriz calcarenítica, típico de ambientes marinos someros del Neógeno (Mioceno), muy comunes en el Algarve portugués.</t>
-  </si>
-  <si>
-    <t>Neógeno</t>
-  </si>
-  <si>
-    <t>Mioceno</t>
-  </si>
-  <si>
-    <t>Parcialmente conservado</t>
-  </si>
-  <si>
-    <t>Gymnospermae</t>
-  </si>
-  <si>
-    <t>Xilópalo</t>
-  </si>
-  <si>
-    <t>Corte transversal de tronco silicificado con preservación detallada del tejido vascular y anillos de crecimiento, testimonio de antiguos bosques mesozoicos del Gondwana.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corte transversal </t>
-  </si>
-  <si>
-    <t>Coniferophytina</t>
-  </si>
-  <si>
-    <t>Araucariales</t>
-  </si>
-  <si>
-    <t>Ejemplar conservado como impresión en caliza, correspondiente a un pez óseo de cuerpo fusiforme, típico de ambientes marinos someros del Cretácico temprano.</t>
-  </si>
-  <si>
-    <t>Pez fósil</t>
-  </si>
-  <si>
-    <t>Diente de tiburón fósil</t>
-  </si>
-  <si>
-    <t>Diente perteneciente a un gran tiburón lamniforme primitivo, antecesor del linaje que culminará en Otodus megalodon. Ejemplar conservado en matriz marina.</t>
-  </si>
-  <si>
-    <t>Trilobite enrollado en posición defensiva, ojos grandes y claramente visibles, con lentes individuales (ojo esquizocroal), cefalón robusto, bien mineralizado, tórax con segmentos marcados y regulares, pigidio relativamente pequeño, exoesqueleto oscuro, calcítico, matriz carbonatada compacta típica del Anti-Atlas.</t>
-  </si>
-  <si>
-    <t>Dimensiones</t>
-  </si>
-  <si>
-    <t>657 gr</t>
-  </si>
-  <si>
-    <t>290 gr</t>
-  </si>
-  <si>
-    <t>30 gr</t>
-  </si>
-  <si>
-    <t>311 gr</t>
-  </si>
-  <si>
-    <t>42 gr</t>
-  </si>
-  <si>
-    <t>516 gr</t>
-  </si>
-  <si>
-    <t>313 gr</t>
-  </si>
-  <si>
-    <t>1,7 Kg</t>
-  </si>
-  <si>
-    <t>2,4 Kg</t>
-  </si>
-  <si>
-    <t>7x10 cm</t>
-  </si>
-  <si>
-    <t>8x8 cm</t>
-  </si>
-  <si>
-    <t>2x5 cm</t>
-  </si>
-  <si>
-    <t>7x9 cm</t>
-  </si>
-  <si>
-    <t>17x25 cm</t>
-  </si>
-  <si>
-    <t>2x6 cm</t>
-  </si>
-  <si>
-    <t>10x18 cm</t>
-  </si>
-  <si>
-    <t>7x13 cm</t>
-  </si>
-  <si>
-    <t>21x14 cm</t>
-  </si>
-  <si>
-    <t>36 gr</t>
-  </si>
-  <si>
-    <t>4x6 cm</t>
-  </si>
-  <si>
-    <t>20 gr</t>
-  </si>
-  <si>
-    <t>2x8</t>
-  </si>
-  <si>
-    <t>Pulido industrial- Cianocrilato</t>
-  </si>
-  <si>
-    <t>87 gr</t>
-  </si>
-  <si>
-    <t>5,5x6,5 cm</t>
-  </si>
-  <si>
-    <t>6,8 × 7 cm</t>
-  </si>
-  <si>
-    <t>Hammatoceras Subinsigne</t>
-  </si>
-  <si>
-    <t>900 gr</t>
-  </si>
-  <si>
-    <t>15x12 cm</t>
-  </si>
-  <si>
-    <t>Mantelliceras sp.</t>
-  </si>
-  <si>
-    <t>2,350 Kg</t>
-  </si>
-  <si>
-    <t>15x18 cm</t>
-  </si>
-  <si>
-    <t>1,5 Kg</t>
-  </si>
-  <si>
-    <t>16x20 cm</t>
-  </si>
-  <si>
-    <t>150 gr</t>
-  </si>
-  <si>
-    <t>10,5x12 cm</t>
-  </si>
-  <si>
-    <t>78 gr</t>
-  </si>
-  <si>
-    <t>605 gr</t>
-  </si>
-  <si>
-    <t>8x5,7 cm</t>
-  </si>
-  <si>
-    <t>12x14 cm</t>
-  </si>
-  <si>
-    <t>270 gr</t>
-  </si>
-  <si>
-    <t>89 gr</t>
-  </si>
-  <si>
-    <t>4,7x10,7 cm</t>
-  </si>
-  <si>
-    <t>8,3x5,2 cm</t>
-  </si>
-  <si>
-    <t>Acadoparadoxides sp.</t>
-  </si>
-  <si>
-    <t>Zona de Zagora (probable)</t>
-  </si>
-  <si>
-    <t>Jurásico superior</t>
-  </si>
-  <si>
-    <t>445 - 460 millones de años</t>
-  </si>
-  <si>
-    <t>Flexicalymene Ouzregui sp.</t>
-  </si>
-  <si>
-    <t>485–500 millones de años</t>
-  </si>
-  <si>
-    <t>Corynexochida</t>
-  </si>
-  <si>
-    <t>Illaenus sp.</t>
-  </si>
-  <si>
-    <t>Yacimientos del río Volkhov (probable)</t>
-  </si>
-  <si>
-    <t>445 - 450 millones de años</t>
-  </si>
-  <si>
-    <t>Género</t>
-  </si>
-  <si>
-    <t>Phacops sp.</t>
-  </si>
-  <si>
-    <t>Región de Alnif</t>
-  </si>
-  <si>
-    <t>Orthoceras sp.</t>
-  </si>
-  <si>
-    <t>360 - 410 millones de años</t>
-  </si>
-  <si>
-    <t>360 - 390 millones de años</t>
-  </si>
-  <si>
-    <t>Región de Erfoud</t>
-  </si>
-  <si>
-    <t>Formaciones de caliza negra del Sahara</t>
-  </si>
-  <si>
-    <t>Jurásico medio</t>
-  </si>
-  <si>
-    <t>Cámbrico medio</t>
-  </si>
-  <si>
-    <t>Ordovícico superior</t>
-  </si>
-  <si>
-    <t>Ordovícico medio</t>
-  </si>
-  <si>
-    <t>Ordovícico tardío</t>
-  </si>
-  <si>
-    <t>Devónico superior</t>
-  </si>
-  <si>
-    <t>460 – 470 millones de años</t>
-  </si>
-  <si>
-    <t>170 - 174 millones de años</t>
-  </si>
-  <si>
-    <t>163 - 166 millones de años</t>
-  </si>
-  <si>
-    <t>94 - 100 millones de años</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Región de </t>
+      <t xml:space="preserve"> o </t>
     </r>
     <r>
       <rPr>
@@ -959,33 +945,33 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Agadir</t>
-    </r>
-    <r>
-      <rPr>
+      <t>Erfoud</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Región de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> o </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
+      <t>Agadir</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Erfoud</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Región de </t>
+      <t xml:space="preserve"> o </t>
     </r>
     <r>
       <rPr>
@@ -996,109 +982,112 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Agadir</t>
-    </r>
-    <r>
-      <rPr>
+      <t>Hamada du Guir</t>
+    </r>
+  </si>
+  <si>
+    <t>100 - 113 millones de años</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cuenca de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> o </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
+      <t>Majunga</t>
+    </r>
+  </si>
+  <si>
+    <t>Madagascar</t>
+  </si>
+  <si>
+    <t>Pteridopsida</t>
+  </si>
+  <si>
+    <t>295 - 310 millones de años</t>
+  </si>
+  <si>
+    <t>Polypodiidae</t>
+  </si>
+  <si>
+    <t>Pecopteris</t>
+  </si>
+  <si>
+    <t>Flexicalymene sp.</t>
+  </si>
+  <si>
+    <t>Quenstedtoceras sp.</t>
+  </si>
+  <si>
+    <t>Cleoniceras sp.</t>
+  </si>
+  <si>
+    <t>5 - 20 millones de años</t>
+  </si>
+  <si>
+    <t>Triásico</t>
+  </si>
+  <si>
+    <t>225 - 250 millones de años</t>
+  </si>
+  <si>
+    <t>Triásico medio</t>
+  </si>
+  <si>
+    <t>Crossognathiformes</t>
+  </si>
+  <si>
+    <t>Cuenca de Araripe</t>
+  </si>
+  <si>
+    <t>Eoceno</t>
+  </si>
+  <si>
+    <t>50 millones de años</t>
+  </si>
+  <si>
+    <t>Ulad Abdun (Khouribga)</t>
+  </si>
+  <si>
+    <t>Otodus obliquus</t>
+  </si>
+  <si>
+    <t>Ejemplar de ammonite planiespiral, con enrollamiento evoluto y ombligo amplio. La concha presenta costulación radial fuerte y densa, con costillas simples que se bifurcan hacia el borde externo, un rasgo diagnóstico del grupo. El relieve costal se conserva bien, aunque con desgaste parcial en algunos sectores. Se observan variaciones cromáticas naturales (grises, ocres y rojizos) debidas a procesos de diagénesis ferruginosa en la matriz calcárea. El área ventral aparece redondeada, sin quilla marcada. El tamaño y robustez sugieren un ejemplar adulto o subadulto.</t>
+  </si>
+  <si>
+    <r>
+      <t>Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Hamada du Guir</t>
-    </r>
-  </si>
-  <si>
-    <t>100 - 113 millones de años</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Cuenca de </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Majunga</t>
-    </r>
-  </si>
-  <si>
-    <t>Madagascar</t>
-  </si>
-  <si>
-    <t>Pteridopsida</t>
-  </si>
-  <si>
-    <t>295 - 310 millones de años</t>
-  </si>
-  <si>
-    <t>Polypodiidae</t>
-  </si>
-  <si>
-    <t>Pecopteris</t>
-  </si>
-  <si>
-    <t>Flexicalymene sp.</t>
-  </si>
-  <si>
-    <t>Quenstedtoceras sp.</t>
-  </si>
-  <si>
-    <t>Cleoniceras sp.</t>
-  </si>
-  <si>
-    <t>5 - 20 millones de años</t>
-  </si>
-  <si>
-    <t>Triásico</t>
-  </si>
-  <si>
-    <t>225 - 250 millones de años</t>
-  </si>
-  <si>
-    <t>Triásico medio</t>
-  </si>
-  <si>
-    <t>Crossognathiformes</t>
-  </si>
-  <si>
-    <t>Cuenca de Araripe</t>
-  </si>
-  <si>
-    <t>Eoceno</t>
-  </si>
-  <si>
-    <t>50 millones de años</t>
-  </si>
-  <si>
-    <t>Ulad Abdun (Khouribga)</t>
-  </si>
-  <si>
-    <t>Otodus obliquus</t>
+      <t>. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Jurásico medio y constituye un importante fósil guía para este intervalo.</t>
+    </r>
+  </si>
+  <si>
+    <t>Ammonite de concha planiespiral evoluta, caracterizada por costillas gruesas y regulares que alcanzan el margen externo, donde forman un contorno dentado. Pertenece al género Mantelliceras, un grupo típico del Cretácico superior, ampliamente utilizado como fósil guía del Cenomaniense. Conservado en matriz calcárea con alteraciones ferruginosas, procedente de depósitos marinos someros del norte de África.</t>
+  </si>
+  <si>
+    <t>Ammonite del Cretácico inferior con concha planiespiral evoluta. El pulido revela la compleja red de suturas internas, correspondientes a los tabiques que separaban las cámaras de flotación. Estas estructuras permitían al animal regular su posición en la columna de agua.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1116,14 +1105,6 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1533,7 +1514,7 @@
         <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1551,7 +1532,7 @@
         <v>2</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1589,19 +1570,19 @@
         <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D2" t="s">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="G2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
@@ -1642,28 +1623,28 @@
         <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="F3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="G3" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H3" t="s">
         <v>10</v>
       </c>
       <c r="I3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="K3" t="s">
         <v>67</v>
@@ -1695,28 +1676,28 @@
         <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="F4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="G4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="H4" t="s">
         <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="J4" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="K4" t="s">
         <v>67</v>
@@ -1725,7 +1706,7 @@
         <v>13</v>
       </c>
       <c r="N4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="O4" t="s">
         <v>83</v>
@@ -1748,28 +1729,28 @@
         <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F5" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="G5" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="H5" t="s">
         <v>10</v>
       </c>
       <c r="I5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="J5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="K5" t="s">
         <v>67</v>
@@ -1801,28 +1782,28 @@
         <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D6" t="s">
         <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="F6" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G6" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H6" t="s">
         <v>10</v>
       </c>
       <c r="I6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="J6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="K6" t="s">
         <v>67</v>
@@ -1834,7 +1815,7 @@
         <v>70</v>
       </c>
       <c r="O6" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="P6" t="s">
         <v>82</v>
@@ -1854,28 +1835,28 @@
         <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D7" t="s">
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F7" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="G7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="H7" t="s">
         <v>10</v>
       </c>
       <c r="I7" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="J7" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="K7" t="s">
         <v>67</v>
@@ -1907,7 +1888,7 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D8" t="s">
         <v>85</v>
@@ -1916,19 +1897,19 @@
         <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H8" t="s">
         <v>10</v>
       </c>
       <c r="I8" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="J8" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="K8" t="s">
         <v>91</v>
@@ -1963,7 +1944,7 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D9" t="s">
         <v>85</v>
@@ -1972,19 +1953,19 @@
         <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G9" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H9" t="s">
         <v>10</v>
       </c>
       <c r="I9" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="J9" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="K9" t="s">
         <v>91</v>
@@ -2019,7 +2000,7 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D10" t="s">
         <v>85</v>
@@ -2028,19 +2009,19 @@
         <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G10" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H10" t="s">
         <v>10</v>
       </c>
       <c r="I10" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="J10" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="K10" t="s">
         <v>91</v>
@@ -2075,7 +2056,7 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D11" t="s">
         <v>85</v>
@@ -2084,19 +2065,19 @@
         <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G11" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="H11" t="s">
         <v>10</v>
       </c>
       <c r="I11" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="J11" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="K11" t="s">
         <v>91</v>
@@ -2131,7 +2112,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D12" t="s">
         <v>85</v>
@@ -2140,19 +2121,19 @@
         <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G12" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H12" t="s">
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J12" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="K12" t="s">
         <v>91</v>
@@ -2187,7 +2168,7 @@
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D13" t="s">
         <v>85</v>
@@ -2196,19 +2177,19 @@
         <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="G13" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H13" t="s">
         <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="J13" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="K13" t="s">
         <v>91</v>
@@ -2232,7 +2213,7 @@
         <v>81</v>
       </c>
       <c r="R13" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -2240,19 +2221,19 @@
         <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D14" t="s">
         <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F14" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
@@ -2261,10 +2242,10 @@
         <v>20</v>
       </c>
       <c r="I14" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="J14" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="K14" t="s">
         <v>91</v>
@@ -2279,7 +2260,7 @@
         <v>24</v>
       </c>
       <c r="O14" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="P14" t="s">
         <v>82</v>
@@ -2296,28 +2277,28 @@
         <v>58</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D15" t="s">
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="F15" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="G15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H15" t="s">
         <v>22</v>
       </c>
       <c r="I15" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="J15" t="s">
         <v>23</v>
@@ -2335,7 +2316,7 @@
         <v>24</v>
       </c>
       <c r="O15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P15" t="s">
         <v>82</v>
@@ -2352,31 +2333,31 @@
         <v>59</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C16" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D16" t="s">
         <v>37</v>
       </c>
       <c r="E16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F16" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="G16" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="H16" t="s">
         <v>10</v>
       </c>
       <c r="I16" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="J16" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="K16" t="s">
         <v>91</v>
@@ -2391,7 +2372,7 @@
         <v>24</v>
       </c>
       <c r="O16" t="s">
-        <v>103</v>
+        <v>222</v>
       </c>
       <c r="P16" t="s">
         <v>82</v>
@@ -2408,31 +2389,31 @@
         <v>60</v>
       </c>
       <c r="B17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D17" t="s">
         <v>37</v>
       </c>
       <c r="E17" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F17" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="G17" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="H17" t="s">
         <v>10</v>
       </c>
       <c r="I17" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="J17" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="K17" t="s">
         <v>91</v>
@@ -2447,7 +2428,7 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>105</v>
+        <v>223</v>
       </c>
       <c r="P17" t="s">
         <v>82</v>
@@ -2464,31 +2445,31 @@
         <v>61</v>
       </c>
       <c r="B18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
       </c>
       <c r="E18" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F18" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="G18" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="H18" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="I18" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="J18" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="K18" t="s">
         <v>91</v>
@@ -2503,7 +2484,7 @@
         <v>24</v>
       </c>
       <c r="O18" t="s">
-        <v>107</v>
+        <v>224</v>
       </c>
       <c r="P18" t="s">
         <v>82</v>
@@ -2520,19 +2501,19 @@
         <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C19" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F19" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="G19" t="s">
         <v>26</v>
@@ -2541,25 +2522,25 @@
         <v>27</v>
       </c>
       <c r="I19" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="J19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="K19" t="s">
         <v>28</v>
       </c>
       <c r="L19" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="M19" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="N19" t="s">
         <v>35</v>
       </c>
       <c r="O19" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="P19" t="s">
         <v>82</v>
@@ -2576,19 +2557,19 @@
         <v>63</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C20" t="s">
+        <v>109</v>
+      </c>
+      <c r="D20" t="s">
+        <v>112</v>
+      </c>
+      <c r="E20" t="s">
         <v>113</v>
       </c>
-      <c r="D20" t="s">
-        <v>116</v>
-      </c>
-      <c r="E20" t="s">
-        <v>117</v>
-      </c>
       <c r="F20" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -2597,31 +2578,31 @@
         <v>31</v>
       </c>
       <c r="I20" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J20" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="K20" t="s">
         <v>91</v>
       </c>
       <c r="L20" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="M20" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="N20" t="s">
         <v>91</v>
       </c>
       <c r="O20" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="P20" t="s">
         <v>82</v>
       </c>
       <c r="Q20" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="R20" t="s">
         <v>77</v>
@@ -2632,19 +2613,19 @@
         <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C21" t="s">
         <v>32</v>
       </c>
       <c r="D21" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E21" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F21" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="G21" t="s">
         <v>33</v>
@@ -2653,28 +2634,28 @@
         <v>34</v>
       </c>
       <c r="I21" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="J21" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="K21" t="s">
         <v>28</v>
       </c>
       <c r="L21" t="s">
+        <v>115</v>
+      </c>
+      <c r="M21" t="s">
         <v>119</v>
       </c>
-      <c r="M21" t="s">
-        <v>123</v>
-      </c>
       <c r="N21" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="O21" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="P21" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="Q21" t="s">
         <v>81</v>
@@ -2688,7 +2669,7 @@
         <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
@@ -2697,22 +2678,22 @@
         <v>37</v>
       </c>
       <c r="E22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F22" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="G22" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="H22" t="s">
         <v>34</v>
       </c>
       <c r="I22" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="J22" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="K22" t="s">
         <v>38</v>
@@ -2724,10 +2705,10 @@
         <v>40</v>
       </c>
       <c r="N22" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="O22" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="P22" t="s">
         <v>82</v>
@@ -2744,31 +2725,31 @@
         <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C23" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="F23" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="G23" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="H23" t="s">
         <v>10</v>
       </c>
       <c r="I23" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J23" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="K23" t="s">
         <v>38</v>
@@ -2783,7 +2764,7 @@
         <v>43</v>
       </c>
       <c r="O23" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="P23" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Nueva actualización de descripción en F-016 (Limonita y bivalvos)
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pascual\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3B1FCC-3B12-40F2-9B40-10B026081864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADD9958-2745-44AB-B37E-C0B8F0557A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1077,10 +1077,10 @@
     </r>
   </si>
   <si>
-    <t>Ammonite de concha planiespiral evoluta, caracterizada por costillas gruesas y regulares que alcanzan el margen externo, donde forman un contorno dentado. Pertenece al género Mantelliceras, un grupo típico del Cretácico superior, ampliamente utilizado como fósil guía del Cenomaniense. Conservado en matriz calcárea con alteraciones ferruginosas, procedente de depósitos marinos someros del norte de África.</t>
-  </si>
-  <si>
     <t>Ammonite del Cretácico inferior con concha planiespiral evoluta. El pulido revela la compleja red de suturas internas, correspondientes a los tabiques que separaban las cámaras de flotación. Estas estructuras permitían al animal regular su posición en la columna de agua.</t>
+  </si>
+  <si>
+    <t>Ammonite caracterizado por una concha de enrollamiento evoluto y una ornamentación robusta de costillas radiales simples. El ejemplar presenta una preservación en matriz margo-caliza con una notable mineralización en limonita, responsable de su coloración ferruginosa. La matriz incluye restos fragmentarios de bivalvos (Ostreida), evidenciando un antiguo ecosistema de plataforma marina somera.</t>
   </si>
 </sst>
 </file>
@@ -2428,7 +2428,7 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="P17" t="s">
         <v>82</v>
@@ -2484,7 +2484,7 @@
         <v>24</v>
       </c>
       <c r="O18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="P18" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Actualizacion de catalogo: Correccion ficha F-015
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pascual\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coleccion Fósiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADD9958-2745-44AB-B37E-C0B8F0557A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04710D66-3F09-4369-889B-2ACB2E62B84D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1062,25 +1062,13 @@
     <t>Ejemplar de ammonite planiespiral, con enrollamiento evoluto y ombligo amplio. La concha presenta costulación radial fuerte y densa, con costillas simples que se bifurcan hacia el borde externo, un rasgo diagnóstico del grupo. El relieve costal se conserva bien, aunque con desgaste parcial en algunos sectores. Se observan variaciones cromáticas naturales (grises, ocres y rojizos) debidas a procesos de diagénesis ferruginosa en la matriz calcárea. El área ventral aparece redondeada, sin quilla marcada. El tamaño y robustez sugieren un ejemplar adulto o subadulto.</t>
   </si>
   <si>
-    <r>
-      <t>Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Jurásico medio y constituye un importante fósil guía para este intervalo.</t>
-    </r>
-  </si>
-  <si>
     <t>Ammonite del Cretácico inferior con concha planiespiral evoluta. El pulido revela la compleja red de suturas internas, correspondientes a los tabiques que separaban las cámaras de flotación. Estas estructuras permitían al animal regular su posición en la columna de agua.</t>
   </si>
   <si>
     <t>Ammonite caracterizado por una concha de enrollamiento evoluto y una ornamentación robusta de costillas radiales simples. El ejemplar presenta una preservación en matriz margo-caliza con una notable mineralización en limonita, responsable de su coloración ferruginosa. La matriz incluye restos fragmentarios de bivalvos (Ostreida), evidenciando un antiguo ecosistema de plataforma marina somera.</t>
+  </si>
+  <si>
+    <t>Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Cretácico superior y constituye un importante fósil guía para este intervalo.</t>
   </si>
 </sst>
 </file>
@@ -2372,7 +2360,7 @@
         <v>24</v>
       </c>
       <c r="O16" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="P16" t="s">
         <v>82</v>
@@ -2428,7 +2416,7 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="P17" t="s">
         <v>82</v>
@@ -2484,7 +2472,7 @@
         <v>24</v>
       </c>
       <c r="O18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="P18" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Actualizacion de catalogo y datos de F-014 desde Excel
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coleccion Fósiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04710D66-3F09-4369-889B-2ACB2E62B84D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB817767-AC66-41B3-A210-4C5A78ABB6AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -615,9 +615,6 @@
     <t>Ammonite</t>
   </si>
   <si>
-    <t>Conjunto fósil formado por dos ammonites asociados, parcialmente superpuestos, conservados en una matriz compacta. Las conchas presentan enrollamiento planiespiral evoluto, con ombligo amplio y costulación radial fina y regular, rasgos característicos del género Dactylioceras. La superficie muestra una piritización parcial a generalizada, visible como áreas de brillo metálico dorado y tonos iridiscentes, especialmente en la matriz y en sectores de la concha. Este tipo de preservación indica enterramiento rápido en condiciones pobres en oxígeno, favoreciendo la sustitución mineral de los tejidos carbonatados. La coexistencia de dos individuos sugiere un evento de acumulación rápida, posiblemente ligado a mortalidad masiva o a corrientes de fondo suaves.</t>
-  </si>
-  <si>
     <t>Cuenca del Volga (probable)</t>
   </si>
   <si>
@@ -904,9 +901,6 @@
   </si>
   <si>
     <t>170 - 174 millones de años</t>
-  </si>
-  <si>
-    <t>163 - 166 millones de años</t>
   </si>
   <si>
     <t>94 - 100 millones de años</t>
@@ -1069,6 +1063,12 @@
   </si>
   <si>
     <t>Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Cretácico superior y constituye un importante fósil guía para este intervalo.</t>
+  </si>
+  <si>
+    <t>Conjunto fósil formado por dos ammonites asociados, parcialmente superpuestos, conservados en una matriz compacta. Las conchas presentan enrollamiento planiespiral evoluto, con ombligo amplio y costulación radial fina y regular, rasgos característicos del género Quenstedtoceras. La superficie muestra una piritización parcial a generalizada, visible como áreas de brillo metálico dorado y tonos iridiscentes, especialmente en la matriz y en sectores de la concha. Este tipo de preservación indica enterramiento rápido en condiciones pobres en oxígeno, favoreciendo la sustitución mineral de los tejidos carbonatados. La coexistencia de dos individuos sugiere un evento de acumulación rápida, posiblemente ligado a mortalidad masiva o a corrientes de fondo suaves.</t>
+  </si>
+  <si>
+    <t>160 - 165 millones de años</t>
   </si>
 </sst>
 </file>
@@ -1502,7 +1502,7 @@
         <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1520,7 +1520,7 @@
         <v>2</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1558,19 +1558,19 @@
         <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D2" t="s">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
@@ -1611,28 +1611,28 @@
         <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H3" t="s">
         <v>10</v>
       </c>
       <c r="I3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K3" t="s">
         <v>67</v>
@@ -1664,28 +1664,28 @@
         <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H4" t="s">
         <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K4" t="s">
         <v>67</v>
@@ -1694,7 +1694,7 @@
         <v>13</v>
       </c>
       <c r="N4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="O4" t="s">
         <v>83</v>
@@ -1717,28 +1717,28 @@
         <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H5" t="s">
         <v>10</v>
       </c>
       <c r="I5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K5" t="s">
         <v>67</v>
@@ -1770,28 +1770,28 @@
         <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D6" t="s">
         <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G6" t="s">
         <v>186</v>
-      </c>
-      <c r="G6" t="s">
-        <v>187</v>
       </c>
       <c r="H6" t="s">
         <v>10</v>
       </c>
       <c r="I6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K6" t="s">
         <v>67</v>
@@ -1803,7 +1803,7 @@
         <v>70</v>
       </c>
       <c r="O6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P6" t="s">
         <v>82</v>
@@ -1823,28 +1823,28 @@
         <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D7" t="s">
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H7" t="s">
         <v>10</v>
       </c>
       <c r="I7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K7" t="s">
         <v>67</v>
@@ -1876,7 +1876,7 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D8" t="s">
         <v>85</v>
@@ -1885,19 +1885,19 @@
         <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H8" t="s">
         <v>10</v>
       </c>
       <c r="I8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K8" t="s">
         <v>91</v>
@@ -1932,7 +1932,7 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D9" t="s">
         <v>85</v>
@@ -1941,19 +1941,19 @@
         <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H9" t="s">
         <v>10</v>
       </c>
       <c r="I9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K9" t="s">
         <v>91</v>
@@ -1988,7 +1988,7 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D10" t="s">
         <v>85</v>
@@ -1997,19 +1997,19 @@
         <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H10" t="s">
         <v>10</v>
       </c>
       <c r="I10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K10" t="s">
         <v>91</v>
@@ -2044,7 +2044,7 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D11" t="s">
         <v>85</v>
@@ -2053,19 +2053,19 @@
         <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H11" t="s">
         <v>10</v>
       </c>
       <c r="I11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K11" t="s">
         <v>91</v>
@@ -2100,7 +2100,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D12" t="s">
         <v>85</v>
@@ -2109,19 +2109,19 @@
         <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H12" t="s">
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K12" t="s">
         <v>91</v>
@@ -2156,7 +2156,7 @@
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D13" t="s">
         <v>85</v>
@@ -2165,19 +2165,19 @@
         <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H13" t="s">
         <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J13" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K13" t="s">
         <v>91</v>
@@ -2201,7 +2201,7 @@
         <v>81</v>
       </c>
       <c r="R13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -2212,16 +2212,16 @@
         <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D14" t="s">
         <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
@@ -2230,10 +2230,10 @@
         <v>20</v>
       </c>
       <c r="I14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K14" t="s">
         <v>91</v>
@@ -2248,7 +2248,7 @@
         <v>24</v>
       </c>
       <c r="O14" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="P14" t="s">
         <v>82</v>
@@ -2268,25 +2268,25 @@
         <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D15" t="s">
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F15" t="s">
-        <v>197</v>
+        <v>224</v>
       </c>
       <c r="G15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H15" t="s">
         <v>22</v>
       </c>
       <c r="I15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J15" t="s">
         <v>23</v>
@@ -2304,7 +2304,7 @@
         <v>24</v>
       </c>
       <c r="O15" t="s">
-        <v>100</v>
+        <v>223</v>
       </c>
       <c r="P15" t="s">
         <v>82</v>
@@ -2324,28 +2324,28 @@
         <v>99</v>
       </c>
       <c r="C16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D16" t="s">
         <v>37</v>
       </c>
       <c r="E16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F16" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="G16" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H16" t="s">
         <v>10</v>
       </c>
       <c r="I16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J16" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K16" t="s">
         <v>91</v>
@@ -2360,7 +2360,7 @@
         <v>24</v>
       </c>
       <c r="O16" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="P16" t="s">
         <v>82</v>
@@ -2380,28 +2380,28 @@
         <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D17" t="s">
         <v>37</v>
       </c>
       <c r="E17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F17" t="s">
+        <v>196</v>
+      </c>
+      <c r="G17" t="s">
         <v>198</v>
-      </c>
-      <c r="G17" t="s">
-        <v>200</v>
       </c>
       <c r="H17" t="s">
         <v>10</v>
       </c>
       <c r="I17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K17" t="s">
         <v>91</v>
@@ -2416,7 +2416,7 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="P17" t="s">
         <v>82</v>
@@ -2436,28 +2436,28 @@
         <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
       </c>
       <c r="E18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F18" t="s">
+        <v>199</v>
+      </c>
+      <c r="G18" t="s">
+        <v>200</v>
+      </c>
+      <c r="H18" t="s">
         <v>201</v>
       </c>
-      <c r="G18" t="s">
-        <v>202</v>
-      </c>
-      <c r="H18" t="s">
-        <v>203</v>
-      </c>
       <c r="I18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K18" t="s">
         <v>91</v>
@@ -2472,7 +2472,7 @@
         <v>24</v>
       </c>
       <c r="O18" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="P18" t="s">
         <v>82</v>
@@ -2489,19 +2489,19 @@
         <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C19" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F19" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="G19" t="s">
         <v>26</v>
@@ -2510,25 +2510,25 @@
         <v>27</v>
       </c>
       <c r="I19" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K19" t="s">
         <v>28</v>
       </c>
       <c r="L19" t="s">
+        <v>202</v>
+      </c>
+      <c r="M19" t="s">
         <v>204</v>
-      </c>
-      <c r="M19" t="s">
-        <v>206</v>
       </c>
       <c r="N19" t="s">
         <v>35</v>
       </c>
       <c r="O19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P19" t="s">
         <v>82</v>
@@ -2545,19 +2545,19 @@
         <v>63</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D20" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20" t="s">
         <v>112</v>
       </c>
-      <c r="E20" t="s">
-        <v>113</v>
-      </c>
       <c r="F20" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -2566,31 +2566,31 @@
         <v>31</v>
       </c>
       <c r="I20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J20" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K20" t="s">
         <v>91</v>
       </c>
       <c r="L20" t="s">
+        <v>106</v>
+      </c>
+      <c r="M20" t="s">
         <v>107</v>
-      </c>
-      <c r="M20" t="s">
-        <v>108</v>
       </c>
       <c r="N20" t="s">
         <v>91</v>
       </c>
       <c r="O20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P20" t="s">
         <v>82</v>
       </c>
       <c r="Q20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="R20" t="s">
         <v>77</v>
@@ -2601,19 +2601,19 @@
         <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C21" t="s">
         <v>32</v>
       </c>
       <c r="D21" t="s">
+        <v>210</v>
+      </c>
+      <c r="E21" t="s">
         <v>212</v>
       </c>
-      <c r="E21" t="s">
-        <v>214</v>
-      </c>
       <c r="F21" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="G21" t="s">
         <v>33</v>
@@ -2622,28 +2622,28 @@
         <v>34</v>
       </c>
       <c r="I21" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J21" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K21" t="s">
         <v>28</v>
       </c>
       <c r="L21" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M21" t="s">
+        <v>118</v>
+      </c>
+      <c r="N21" t="s">
         <v>119</v>
       </c>
-      <c r="N21" t="s">
-        <v>120</v>
-      </c>
       <c r="O21" t="s">
+        <v>116</v>
+      </c>
+      <c r="P21" t="s">
         <v>117</v>
-      </c>
-      <c r="P21" t="s">
-        <v>118</v>
       </c>
       <c r="Q21" t="s">
         <v>81</v>
@@ -2657,7 +2657,7 @@
         <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
@@ -2666,22 +2666,22 @@
         <v>37</v>
       </c>
       <c r="E22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F22" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G22" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H22" t="s">
         <v>34</v>
       </c>
       <c r="I22" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J22" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K22" t="s">
         <v>38</v>
@@ -2693,10 +2693,10 @@
         <v>40</v>
       </c>
       <c r="N22" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="O22" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P22" t="s">
         <v>82</v>
@@ -2713,31 +2713,31 @@
         <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C23" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
       <c r="E23" t="s">
+        <v>215</v>
+      </c>
+      <c r="F23" t="s">
+        <v>216</v>
+      </c>
+      <c r="G23" t="s">
         <v>217</v>
-      </c>
-      <c r="F23" t="s">
-        <v>218</v>
-      </c>
-      <c r="G23" t="s">
-        <v>219</v>
       </c>
       <c r="H23" t="s">
         <v>10</v>
       </c>
       <c r="I23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K23" t="s">
         <v>38</v>
@@ -2752,7 +2752,7 @@
         <v>43</v>
       </c>
       <c r="O23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="P23" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Actualización de catálogo y nuevas imágenes para F-023
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coleccion Fósiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pascual\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB817767-AC66-41B3-A210-4C5A78ABB6AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C87E0DF-5912-4913-9BE3-DA28A24E067F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="235">
   <si>
     <t>Periodo</t>
   </si>
@@ -615,6 +615,9 @@
     <t>Ammonite</t>
   </si>
   <si>
+    <t>Conjunto fósil formado por dos ammonites asociados, parcialmente superpuestos, conservados en una matriz compacta. Las conchas presentan enrollamiento planiespiral evoluto, con ombligo amplio y costulación radial fina y regular, rasgos característicos del género Dactylioceras. La superficie muestra una piritización parcial a generalizada, visible como áreas de brillo metálico dorado y tonos iridiscentes, especialmente en la matriz y en sectores de la concha. Este tipo de preservación indica enterramiento rápido en condiciones pobres en oxígeno, favoreciendo la sustitución mineral de los tejidos carbonatados. La coexistencia de dos individuos sugiere un evento de acumulación rápida, posiblemente ligado a mortalidad masiva o a corrientes de fondo suaves.</t>
+  </si>
+  <si>
     <t>Cuenca del Volga (probable)</t>
   </si>
   <si>
@@ -901,6 +904,9 @@
   </si>
   <si>
     <t>170 - 174 millones de años</t>
+  </si>
+  <si>
+    <t>163 - 166 millones de años</t>
   </si>
   <si>
     <t>94 - 100 millones de años</t>
@@ -1056,19 +1062,67 @@
     <t>Ejemplar de ammonite planiespiral, con enrollamiento evoluto y ombligo amplio. La concha presenta costulación radial fuerte y densa, con costillas simples que se bifurcan hacia el borde externo, un rasgo diagnóstico del grupo. El relieve costal se conserva bien, aunque con desgaste parcial en algunos sectores. Se observan variaciones cromáticas naturales (grises, ocres y rojizos) debidas a procesos de diagénesis ferruginosa en la matriz calcárea. El área ventral aparece redondeada, sin quilla marcada. El tamaño y robustez sugieren un ejemplar adulto o subadulto.</t>
   </si>
   <si>
+    <r>
+      <t>Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Jurásico medio y constituye un importante fósil guía para este intervalo.</t>
+    </r>
+  </si>
+  <si>
     <t>Ammonite del Cretácico inferior con concha planiespiral evoluta. El pulido revela la compleja red de suturas internas, correspondientes a los tabiques que separaban las cámaras de flotación. Estas estructuras permitían al animal regular su posición en la columna de agua.</t>
   </si>
   <si>
     <t>Ammonite caracterizado por una concha de enrollamiento evoluto y una ornamentación robusta de costillas radiales simples. El ejemplar presenta una preservación en matriz margo-caliza con una notable mineralización en limonita, responsable de su coloración ferruginosa. La matriz incluye restos fragmentarios de bivalvos (Ostreida), evidenciando un antiguo ecosistema de plataforma marina somera.</t>
   </si>
   <si>
-    <t>Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Cretácico superior y constituye un importante fósil guía para este intervalo.</t>
-  </si>
-  <si>
-    <t>Conjunto fósil formado por dos ammonites asociados, parcialmente superpuestos, conservados en una matriz compacta. Las conchas presentan enrollamiento planiespiral evoluto, con ombligo amplio y costulación radial fina y regular, rasgos característicos del género Quenstedtoceras. La superficie muestra una piritización parcial a generalizada, visible como áreas de brillo metálico dorado y tonos iridiscentes, especialmente en la matriz y en sectores de la concha. Este tipo de preservación indica enterramiento rápido en condiciones pobres en oxígeno, favoreciendo la sustitución mineral de los tejidos carbonatados. La coexistencia de dos individuos sugiere un evento de acumulación rápida, posiblemente ligado a mortalidad masiva o a corrientes de fondo suaves.</t>
-  </si>
-  <si>
-    <t>160 - 165 millones de años</t>
+    <t>F-023</t>
+  </si>
+  <si>
+    <r>
+      <t>Lopha</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sp.</t>
+    </r>
+  </si>
+  <si>
+    <t>Marruecos (Probable región del Atlas/Erfoud)</t>
+  </si>
+  <si>
+    <t>Bivalvia</t>
+  </si>
+  <si>
+    <t>Ostreida</t>
+  </si>
+  <si>
+    <t>Molusco Bivalvo</t>
+  </si>
+  <si>
+    <t>100-120 millones de años</t>
+  </si>
+  <si>
+    <t>Molusco bivalvo inequivalve caracterizado por una fuerte ornamentación de costillas radiales ramificadas. Presenta una comisura marginal en zigzag (forma de "cresta de gallo") altamente pronunciada. Pieza de excepcional interés por su silicificación. El material biogénico original ha sido sustituido por sílice (calcedonia/microcuarzo), visible en el interior de las valvas por su textura vítrea y fractura concoidea. La matriz residual externa presenta tonalidades ocre típicas de sedimentos calcáreos meteorizados en climas áridos.</t>
+  </si>
+  <si>
+    <t>226 gr</t>
+  </si>
+  <si>
+    <t>7,3x8,1 cm</t>
   </si>
 </sst>
 </file>
@@ -1472,7 +1526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -1502,7 +1556,7 @@
         <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1520,7 +1574,7 @@
         <v>2</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1558,19 +1612,19 @@
         <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D2" t="s">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
@@ -1611,28 +1665,28 @@
         <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H3" t="s">
         <v>10</v>
       </c>
       <c r="I3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K3" t="s">
         <v>67</v>
@@ -1664,28 +1718,28 @@
         <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H4" t="s">
         <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K4" t="s">
         <v>67</v>
@@ -1694,7 +1748,7 @@
         <v>13</v>
       </c>
       <c r="N4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="O4" t="s">
         <v>83</v>
@@ -1717,28 +1771,28 @@
         <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H5" t="s">
         <v>10</v>
       </c>
       <c r="I5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K5" t="s">
         <v>67</v>
@@ -1770,28 +1824,28 @@
         <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D6" t="s">
         <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H6" t="s">
         <v>10</v>
       </c>
       <c r="I6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K6" t="s">
         <v>67</v>
@@ -1803,7 +1857,7 @@
         <v>70</v>
       </c>
       <c r="O6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P6" t="s">
         <v>82</v>
@@ -1823,28 +1877,28 @@
         <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D7" t="s">
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H7" t="s">
         <v>10</v>
       </c>
       <c r="I7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K7" t="s">
         <v>67</v>
@@ -1876,7 +1930,7 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D8" t="s">
         <v>85</v>
@@ -1885,19 +1939,19 @@
         <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H8" t="s">
         <v>10</v>
       </c>
       <c r="I8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K8" t="s">
         <v>91</v>
@@ -1932,7 +1986,7 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D9" t="s">
         <v>85</v>
@@ -1941,19 +1995,19 @@
         <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H9" t="s">
         <v>10</v>
       </c>
       <c r="I9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K9" t="s">
         <v>91</v>
@@ -1988,7 +2042,7 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D10" t="s">
         <v>85</v>
@@ -1997,19 +2051,19 @@
         <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H10" t="s">
         <v>10</v>
       </c>
       <c r="I10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K10" t="s">
         <v>91</v>
@@ -2044,7 +2098,7 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D11" t="s">
         <v>85</v>
@@ -2053,19 +2107,19 @@
         <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H11" t="s">
         <v>10</v>
       </c>
       <c r="I11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K11" t="s">
         <v>91</v>
@@ -2100,7 +2154,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D12" t="s">
         <v>85</v>
@@ -2109,19 +2163,19 @@
         <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G12" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H12" t="s">
         <v>10</v>
       </c>
       <c r="I12" t="s">
+        <v>146</v>
+      </c>
+      <c r="J12" t="s">
         <v>145</v>
-      </c>
-      <c r="J12" t="s">
-        <v>144</v>
       </c>
       <c r="K12" t="s">
         <v>91</v>
@@ -2156,7 +2210,7 @@
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D13" t="s">
         <v>85</v>
@@ -2165,19 +2219,19 @@
         <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H13" t="s">
         <v>10</v>
       </c>
       <c r="I13" t="s">
+        <v>148</v>
+      </c>
+      <c r="J13" t="s">
         <v>147</v>
-      </c>
-      <c r="J13" t="s">
-        <v>146</v>
       </c>
       <c r="K13" t="s">
         <v>91</v>
@@ -2201,7 +2255,7 @@
         <v>81</v>
       </c>
       <c r="R13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -2212,16 +2266,16 @@
         <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D14" t="s">
         <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
@@ -2230,10 +2284,10 @@
         <v>20</v>
       </c>
       <c r="I14" t="s">
+        <v>151</v>
+      </c>
+      <c r="J14" t="s">
         <v>150</v>
-      </c>
-      <c r="J14" t="s">
-        <v>149</v>
       </c>
       <c r="K14" t="s">
         <v>91</v>
@@ -2248,7 +2302,7 @@
         <v>24</v>
       </c>
       <c r="O14" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="P14" t="s">
         <v>82</v>
@@ -2268,25 +2322,25 @@
         <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D15" t="s">
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F15" t="s">
-        <v>224</v>
+        <v>197</v>
       </c>
       <c r="G15" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H15" t="s">
         <v>22</v>
       </c>
       <c r="I15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J15" t="s">
         <v>23</v>
@@ -2304,7 +2358,7 @@
         <v>24</v>
       </c>
       <c r="O15" t="s">
-        <v>223</v>
+        <v>100</v>
       </c>
       <c r="P15" t="s">
         <v>82</v>
@@ -2324,28 +2378,28 @@
         <v>99</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D16" t="s">
         <v>37</v>
       </c>
       <c r="E16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F16" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G16" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="H16" t="s">
         <v>10</v>
       </c>
       <c r="I16" t="s">
+        <v>155</v>
+      </c>
+      <c r="J16" t="s">
         <v>154</v>
-      </c>
-      <c r="J16" t="s">
-        <v>153</v>
       </c>
       <c r="K16" t="s">
         <v>91</v>
@@ -2380,28 +2434,28 @@
         <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D17" t="s">
         <v>37</v>
       </c>
       <c r="E17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F17" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G17" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H17" t="s">
         <v>10</v>
       </c>
       <c r="I17" t="s">
+        <v>158</v>
+      </c>
+      <c r="J17" t="s">
         <v>157</v>
-      </c>
-      <c r="J17" t="s">
-        <v>156</v>
       </c>
       <c r="K17" t="s">
         <v>91</v>
@@ -2416,7 +2470,7 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="P17" t="s">
         <v>82</v>
@@ -2436,28 +2490,28 @@
         <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
       </c>
       <c r="E18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F18" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="G18" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H18" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I18" t="s">
+        <v>160</v>
+      </c>
+      <c r="J18" t="s">
         <v>159</v>
-      </c>
-      <c r="J18" t="s">
-        <v>158</v>
       </c>
       <c r="K18" t="s">
         <v>91</v>
@@ -2472,7 +2526,7 @@
         <v>24</v>
       </c>
       <c r="O18" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="P18" t="s">
         <v>82</v>
@@ -2489,19 +2543,19 @@
         <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C19" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F19" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G19" t="s">
         <v>26</v>
@@ -2510,25 +2564,25 @@
         <v>27</v>
       </c>
       <c r="I19" t="s">
+        <v>162</v>
+      </c>
+      <c r="J19" t="s">
         <v>161</v>
-      </c>
-      <c r="J19" t="s">
-        <v>160</v>
       </c>
       <c r="K19" t="s">
         <v>28</v>
       </c>
       <c r="L19" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="M19" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="N19" t="s">
         <v>35</v>
       </c>
       <c r="O19" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P19" t="s">
         <v>82</v>
@@ -2545,19 +2599,19 @@
         <v>63</v>
       </c>
       <c r="B20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C20" t="s">
         <v>109</v>
       </c>
-      <c r="C20" t="s">
-        <v>108</v>
-      </c>
       <c r="D20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F20" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -2566,31 +2620,31 @@
         <v>31</v>
       </c>
       <c r="I20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K20" t="s">
         <v>91</v>
       </c>
       <c r="L20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N20" t="s">
         <v>91</v>
       </c>
       <c r="O20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P20" t="s">
         <v>82</v>
       </c>
       <c r="Q20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="R20" t="s">
         <v>77</v>
@@ -2601,19 +2655,19 @@
         <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C21" t="s">
         <v>32</v>
       </c>
       <c r="D21" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E21" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F21" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G21" t="s">
         <v>33</v>
@@ -2622,28 +2676,28 @@
         <v>34</v>
       </c>
       <c r="I21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J21" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K21" t="s">
         <v>28</v>
       </c>
       <c r="L21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="M21" t="s">
+        <v>119</v>
+      </c>
+      <c r="N21" t="s">
+        <v>120</v>
+      </c>
+      <c r="O21" t="s">
+        <v>117</v>
+      </c>
+      <c r="P21" t="s">
         <v>118</v>
-      </c>
-      <c r="N21" t="s">
-        <v>119</v>
-      </c>
-      <c r="O21" t="s">
-        <v>116</v>
-      </c>
-      <c r="P21" t="s">
-        <v>117</v>
       </c>
       <c r="Q21" t="s">
         <v>81</v>
@@ -2657,7 +2711,7 @@
         <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
@@ -2666,22 +2720,22 @@
         <v>37</v>
       </c>
       <c r="E22" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F22" t="s">
-        <v>199</v>
+        <v>231</v>
       </c>
       <c r="G22" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="H22" t="s">
         <v>34</v>
       </c>
       <c r="I22" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J22" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K22" t="s">
         <v>38</v>
@@ -2693,10 +2747,10 @@
         <v>40</v>
       </c>
       <c r="N22" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="O22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="P22" t="s">
         <v>82</v>
@@ -2713,31 +2767,31 @@
         <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C23" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F23" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G23" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="H23" t="s">
         <v>10</v>
       </c>
       <c r="I23" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K23" t="s">
         <v>38</v>
@@ -2752,7 +2806,7 @@
         <v>43</v>
       </c>
       <c r="O23" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P23" t="s">
         <v>82</v>
@@ -2761,6 +2815,59 @@
         <v>81</v>
       </c>
       <c r="R23" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>225</v>
+      </c>
+      <c r="B24" t="s">
+        <v>230</v>
+      </c>
+      <c r="C24" t="s">
+        <v>226</v>
+      </c>
+      <c r="D24" t="s">
+        <v>37</v>
+      </c>
+      <c r="E24" t="s">
+        <v>103</v>
+      </c>
+      <c r="F24" t="s">
+        <v>231</v>
+      </c>
+      <c r="G24" t="s">
+        <v>227</v>
+      </c>
+      <c r="H24" t="s">
+        <v>10</v>
+      </c>
+      <c r="I24" t="s">
+        <v>234</v>
+      </c>
+      <c r="J24" t="s">
+        <v>233</v>
+      </c>
+      <c r="K24" t="s">
+        <v>91</v>
+      </c>
+      <c r="L24" t="s">
+        <v>228</v>
+      </c>
+      <c r="N24" t="s">
+        <v>229</v>
+      </c>
+      <c r="O24" t="s">
+        <v>232</v>
+      </c>
+      <c r="P24" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>81</v>
+      </c>
+      <c r="R24" t="s">
         <v>77</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza catalogo de fosiles desde Excel y sincroniza JSON
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pascual\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coleccion Fósiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C87E0DF-5912-4913-9BE3-DA28A24E067F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61089FFE-6FC2-4630-87CB-394768505AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="232">
   <si>
     <t>Periodo</t>
   </si>
@@ -855,9 +855,6 @@
     <t>Yacimientos del río Volkhov (probable)</t>
   </si>
   <si>
-    <t>445 - 450 millones de años</t>
-  </si>
-  <si>
     <t>Género</t>
   </si>
   <si>
@@ -894,22 +891,10 @@
     <t>Ordovícico medio</t>
   </si>
   <si>
-    <t>Ordovícico tardío</t>
-  </si>
-  <si>
     <t>Devónico superior</t>
   </si>
   <si>
     <t>460 – 470 millones de años</t>
-  </si>
-  <si>
-    <t>170 - 174 millones de años</t>
-  </si>
-  <si>
-    <t>163 - 166 millones de años</t>
-  </si>
-  <si>
-    <t>94 - 100 millones de años</t>
   </si>
   <si>
     <r>
@@ -986,9 +971,6 @@
     </r>
   </si>
   <si>
-    <t>100 - 113 millones de años</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Cuenca de </t>
     </r>
@@ -1011,9 +993,6 @@
     <t>Pteridopsida</t>
   </si>
   <si>
-    <t>295 - 310 millones de años</t>
-  </si>
-  <si>
     <t>Polypodiidae</t>
   </si>
   <si>
@@ -1035,9 +1014,6 @@
     <t>Triásico</t>
   </si>
   <si>
-    <t>225 - 250 millones de años</t>
-  </si>
-  <si>
     <t>Triásico medio</t>
   </si>
   <si>
@@ -1048,9 +1024,6 @@
   </si>
   <si>
     <t>Eoceno</t>
-  </si>
-  <si>
-    <t>50 millones de años</t>
   </si>
   <si>
     <t>Ulad Abdun (Khouribga)</t>
@@ -1113,9 +1086,6 @@
     <t>Molusco Bivalvo</t>
   </si>
   <si>
-    <t>100-120 millones de años</t>
-  </si>
-  <si>
     <t>Molusco bivalvo inequivalve caracterizado por una fuerte ornamentación de costillas radiales ramificadas. Presenta una comisura marginal en zigzag (forma de "cresta de gallo") altamente pronunciada. Pieza de excepcional interés por su silicificación. El material biogénico original ha sido sustituido por sílice (calcedonia/microcuarzo), visible en el interior de las valvas por su textura vítrea y fractura concoidea. La matriz residual externa presenta tonalidades ocre típicas de sedimentos calcáreos meteorizados en climas áridos.</t>
   </si>
   <si>
@@ -1123,6 +1093,27 @@
   </si>
   <si>
     <t>7,3x8,1 cm</t>
+  </si>
+  <si>
+    <t>160 - 175 millones de años</t>
+  </si>
+  <si>
+    <t>145 - 160 millones de años</t>
+  </si>
+  <si>
+    <t>66 - 100 millones de años</t>
+  </si>
+  <si>
+    <t>100-145 millones de años</t>
+  </si>
+  <si>
+    <t>300 - 307 millones de años</t>
+  </si>
+  <si>
+    <t>235 - 250 millones de años</t>
+  </si>
+  <si>
+    <t>35- 55 millones de años</t>
   </si>
 </sst>
 </file>
@@ -1556,7 +1547,7 @@
         <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1618,7 +1609,7 @@
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F2" t="s">
         <v>176</v>
@@ -1671,13 +1662,13 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F3" t="s">
         <v>174</v>
       </c>
       <c r="G3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H3" t="s">
         <v>10</v>
@@ -1724,10 +1715,10 @@
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F4" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G4" t="s">
         <v>179</v>
@@ -1771,19 +1762,19 @@
         <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="F5" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="G5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H5" t="s">
         <v>10</v>
@@ -1824,19 +1815,19 @@
         <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D6" t="s">
         <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G6" t="s">
         <v>186</v>
-      </c>
-      <c r="G6" t="s">
-        <v>187</v>
       </c>
       <c r="H6" t="s">
         <v>10</v>
@@ -1877,19 +1868,19 @@
         <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D7" t="s">
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="F7" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="G7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H7" t="s">
         <v>10</v>
@@ -1930,7 +1921,7 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D8" t="s">
         <v>85</v>
@@ -1939,10 +1930,10 @@
         <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H8" t="s">
         <v>10</v>
@@ -1986,7 +1977,7 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D9" t="s">
         <v>85</v>
@@ -1995,10 +1986,10 @@
         <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H9" t="s">
         <v>10</v>
@@ -2042,7 +2033,7 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D10" t="s">
         <v>85</v>
@@ -2051,10 +2042,10 @@
         <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H10" t="s">
         <v>10</v>
@@ -2098,7 +2089,7 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D11" t="s">
         <v>85</v>
@@ -2107,10 +2098,10 @@
         <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H11" t="s">
         <v>10</v>
@@ -2154,7 +2145,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D12" t="s">
         <v>85</v>
@@ -2163,10 +2154,10 @@
         <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H12" t="s">
         <v>10</v>
@@ -2210,7 +2201,7 @@
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D13" t="s">
         <v>85</v>
@@ -2219,10 +2210,10 @@
         <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H13" t="s">
         <v>10</v>
@@ -2272,10 +2263,10 @@
         <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F14" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
@@ -2302,7 +2293,7 @@
         <v>24</v>
       </c>
       <c r="O14" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="P14" t="s">
         <v>82</v>
@@ -2322,7 +2313,7 @@
         <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="D15" t="s">
         <v>18</v>
@@ -2331,7 +2322,7 @@
         <v>173</v>
       </c>
       <c r="F15" t="s">
-        <v>197</v>
+        <v>226</v>
       </c>
       <c r="G15" t="s">
         <v>101</v>
@@ -2387,10 +2378,10 @@
         <v>102</v>
       </c>
       <c r="F16" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="G16" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="H16" t="s">
         <v>10</v>
@@ -2414,7 +2405,7 @@
         <v>24</v>
       </c>
       <c r="O16" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="P16" t="s">
         <v>82</v>
@@ -2443,10 +2434,10 @@
         <v>102</v>
       </c>
       <c r="F17" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="G17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="H17" t="s">
         <v>10</v>
@@ -2470,7 +2461,7 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="P17" t="s">
         <v>82</v>
@@ -2490,7 +2481,7 @@
         <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
@@ -2499,13 +2490,13 @@
         <v>103</v>
       </c>
       <c r="F18" t="s">
-        <v>201</v>
+        <v>228</v>
       </c>
       <c r="G18" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="H18" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="I18" t="s">
         <v>160</v>
@@ -2526,7 +2517,7 @@
         <v>24</v>
       </c>
       <c r="O18" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="P18" t="s">
         <v>82</v>
@@ -2546,7 +2537,7 @@
         <v>104</v>
       </c>
       <c r="C19" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
@@ -2555,7 +2546,7 @@
         <v>105</v>
       </c>
       <c r="F19" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="G19" t="s">
         <v>26</v>
@@ -2573,10 +2564,10 @@
         <v>28</v>
       </c>
       <c r="L19" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="M19" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="N19" t="s">
         <v>35</v>
@@ -2611,7 +2602,7 @@
         <v>113</v>
       </c>
       <c r="F20" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -2661,13 +2652,13 @@
         <v>32</v>
       </c>
       <c r="D21" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="E21" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="F21" t="s">
-        <v>213</v>
+        <v>230</v>
       </c>
       <c r="G21" t="s">
         <v>33</v>
@@ -2723,10 +2714,10 @@
         <v>103</v>
       </c>
       <c r="F22" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G22" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="H22" t="s">
         <v>34</v>
@@ -2747,7 +2738,7 @@
         <v>40</v>
       </c>
       <c r="N22" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="O22" t="s">
         <v>121</v>
@@ -2770,19 +2761,19 @@
         <v>123</v>
       </c>
       <c r="C23" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="F23" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="G23" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="H23" t="s">
         <v>10</v>
@@ -2820,13 +2811,13 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B24" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="C24" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="D24" t="s">
         <v>37</v>
@@ -2835,31 +2826,31 @@
         <v>103</v>
       </c>
       <c r="F24" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G24" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="H24" t="s">
         <v>10</v>
       </c>
       <c r="I24" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="J24" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="K24" t="s">
         <v>91</v>
       </c>
       <c r="L24" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="N24" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="O24" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="P24" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
Actualizar catálogo desde Excel (23 fósiles)
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coleccion Fósiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61089FFE-6FC2-4630-87CB-394768505AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E11956B-ADFE-440D-A043-047FE0AE2DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="237">
   <si>
     <t>Periodo</t>
   </si>
@@ -124,16 +124,10 @@
     <t>Psaronius brasiliensis</t>
   </si>
   <si>
-    <t>Maranhao</t>
-  </si>
-  <si>
     <t>Brasil</t>
   </si>
   <si>
     <t>Marattiales</t>
-  </si>
-  <si>
-    <t>Rhacolepis</t>
   </si>
   <si>
     <t>Cretácico</t>
@@ -450,9 +444,6 @@
     <t>Conservación media</t>
   </si>
   <si>
-    <t>Trilobite enrollado en posición defensiva. Ejemplar con exoesqueleto parcialmente conservado, segmentos torácicos bien visibles y cefalón erosionado. Matriz carbonatada.</t>
-  </si>
-  <si>
     <t>Orthocerida</t>
   </si>
   <si>
@@ -666,9 +657,6 @@
     <t>Xilópalo</t>
   </si>
   <si>
-    <t>Corte transversal de tronco silicificado con preservación detallada del tejido vascular y anillos de crecimiento, testimonio de antiguos bosques mesozoicos del Gondwana.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Corte transversal </t>
   </si>
   <si>
@@ -783,9 +771,6 @@
     <t>15x12 cm</t>
   </si>
   <si>
-    <t>Mantelliceras sp.</t>
-  </si>
-  <si>
     <t>2,350 Kg</t>
   </si>
   <si>
@@ -828,12 +813,6 @@
     <t>8,3x5,2 cm</t>
   </si>
   <si>
-    <t>Acadoparadoxides sp.</t>
-  </si>
-  <si>
-    <t>Zona de Zagora (probable)</t>
-  </si>
-  <si>
     <t>Jurásico superior</t>
   </si>
   <si>
@@ -843,9 +822,6 @@
     <t>Flexicalymene Ouzregui sp.</t>
   </si>
   <si>
-    <t>485–500 millones de años</t>
-  </si>
-  <si>
     <t>Corynexochida</t>
   </si>
   <si>
@@ -877,9 +853,6 @@
   </si>
   <si>
     <t>Formaciones de caliza negra del Sahara</t>
-  </si>
-  <si>
-    <t>Jurásico medio</t>
   </si>
   <si>
     <t>Cámbrico medio</t>
@@ -971,149 +944,179 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Cuenca de </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
+    <t>Pteridopsida</t>
+  </si>
+  <si>
+    <t>Polypodiidae</t>
+  </si>
+  <si>
+    <t>Flexicalymene sp.</t>
+  </si>
+  <si>
+    <t>Quenstedtoceras sp.</t>
+  </si>
+  <si>
+    <t>Cleoniceras sp.</t>
+  </si>
+  <si>
+    <t>5 - 20 millones de años</t>
+  </si>
+  <si>
+    <t>Crossognathiformes</t>
+  </si>
+  <si>
+    <t>Cuenca de Araripe</t>
+  </si>
+  <si>
+    <t>Eoceno</t>
+  </si>
+  <si>
+    <t>Otodus obliquus</t>
+  </si>
+  <si>
+    <t>Ejemplar de ammonite planiespiral, con enrollamiento evoluto y ombligo amplio. La concha presenta costulación radial fuerte y densa, con costillas simples que se bifurcan hacia el borde externo, un rasgo diagnóstico del grupo. El relieve costal se conserva bien, aunque con desgaste parcial en algunos sectores. Se observan variaciones cromáticas naturales (grises, ocres y rojizos) debidas a procesos de diagénesis ferruginosa en la matriz calcárea. El área ventral aparece redondeada, sin quilla marcada. El tamaño y robustez sugieren un ejemplar adulto o subadulto.</t>
+  </si>
+  <si>
+    <t>Ammonite caracterizado por una concha de enrollamiento evoluto y una ornamentación robusta de costillas radiales simples. El ejemplar presenta una preservación en matriz margo-caliza con una notable mineralización en limonita, responsable de su coloración ferruginosa. La matriz incluye restos fragmentarios de bivalvos (Ostreida), evidenciando un antiguo ecosistema de plataforma marina somera.</t>
+  </si>
+  <si>
+    <t>F-023</t>
+  </si>
+  <si>
+    <r>
+      <t>Lopha</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Majunga</t>
-    </r>
-  </si>
-  <si>
-    <t>Madagascar</t>
-  </si>
-  <si>
-    <t>Pteridopsida</t>
-  </si>
-  <si>
-    <t>Polypodiidae</t>
-  </si>
-  <si>
-    <t>Pecopteris</t>
-  </si>
-  <si>
-    <t>Flexicalymene sp.</t>
-  </si>
-  <si>
-    <t>Quenstedtoceras sp.</t>
-  </si>
-  <si>
-    <t>Cleoniceras sp.</t>
-  </si>
-  <si>
-    <t>5 - 20 millones de años</t>
-  </si>
-  <si>
-    <t>Triásico</t>
-  </si>
-  <si>
-    <t>Triásico medio</t>
-  </si>
-  <si>
-    <t>Crossognathiformes</t>
-  </si>
-  <si>
-    <t>Cuenca de Araripe</t>
-  </si>
-  <si>
-    <t>Eoceno</t>
-  </si>
-  <si>
-    <t>Ulad Abdun (Khouribga)</t>
-  </si>
-  <si>
-    <t>Otodus obliquus</t>
-  </si>
-  <si>
-    <t>Ejemplar de ammonite planiespiral, con enrollamiento evoluto y ombligo amplio. La concha presenta costulación radial fuerte y densa, con costillas simples que se bifurcan hacia el borde externo, un rasgo diagnóstico del grupo. El relieve costal se conserva bien, aunque con desgaste parcial en algunos sectores. Se observan variaciones cromáticas naturales (grises, ocres y rojizos) debidas a procesos de diagénesis ferruginosa en la matriz calcárea. El área ventral aparece redondeada, sin quilla marcada. El tamaño y robustez sugieren un ejemplar adulto o subadulto.</t>
-  </si>
-  <si>
-    <r>
-      <t>Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada</t>
-    </r>
-    <r>
-      <rPr>
+      <t xml:space="preserve"> sp.</t>
+    </r>
+  </si>
+  <si>
+    <t>Marruecos (Probable región del Atlas/Erfoud)</t>
+  </si>
+  <si>
+    <t>Bivalvia</t>
+  </si>
+  <si>
+    <t>Ostreida</t>
+  </si>
+  <si>
+    <t>Molusco Bivalvo</t>
+  </si>
+  <si>
+    <t>Molusco bivalvo inequivalve caracterizado por una fuerte ornamentación de costillas radiales ramificadas. Presenta una comisura marginal en zigzag (forma de "cresta de gallo") altamente pronunciada. Pieza de excepcional interés por su silicificación. El material biogénico original ha sido sustituido por sílice (calcedonia/microcuarzo), visible en el interior de las valvas por su textura vítrea y fractura concoidea. La matriz residual externa presenta tonalidades ocre típicas de sedimentos calcáreos meteorizados en climas áridos.</t>
+  </si>
+  <si>
+    <t>226 gr</t>
+  </si>
+  <si>
+    <t>7,3x8,1 cm</t>
+  </si>
+  <si>
+    <t>300 - 307 millones de años</t>
+  </si>
+  <si>
+    <t>Colpocoryphe grandis</t>
+  </si>
+  <si>
+    <t>Ordovícico Medio</t>
+  </si>
+  <si>
+    <t>Región de Zagora</t>
+  </si>
+  <si>
+    <t>Ejemplar con exoesqueleto parcialmente conservado, segmentos torácicos bien visibles y cefalón erosionado. Glabela ancha, con lóbulos laterales bien definidos. El cuerpo tiene una forma más "parabólica" o ancha en los hombros, que se va estrechando de forma constante hacia el pigidio (cola). Matriz carbonatada.</t>
+  </si>
+  <si>
+    <t>Goniatites</t>
+  </si>
+  <si>
+    <t>Goniatitida</t>
+  </si>
+  <si>
+    <t>Goniatites sp.</t>
+  </si>
+  <si>
+    <t>Perisphinctes sp.</t>
+  </si>
+  <si>
+    <t>Alethopteris</t>
+  </si>
+  <si>
+    <t>Ammonite del Devónico con concha planiespiral evoluta. El pulido revela la compleja red de suturas internas, correspondientes a los tabiques que separaban las cámaras de flotación. Estas estructuras permitían al animal regular su posición en la columna de agua.</t>
+  </si>
+  <si>
+    <t>Ammonite de tamaño medio con concha planiespiral evoluta y ombligo amplio. Presenta costulación radial fuerte y bifurcada. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Jurásico superior y constituye un importante fósil guía para este intervalo.</t>
+  </si>
+  <si>
+    <t>Pérmico</t>
+  </si>
+  <si>
+    <t>Pérmico Inferior</t>
+  </si>
+  <si>
+    <t>270 - 295 millones de años</t>
+  </si>
+  <si>
+    <t>Bosque petrificado de Araguaína, Maranhao</t>
+  </si>
+  <si>
+    <t>Helecho arborescente extinto. Se observa un manto de raíces adventicias. Como estos helechos no tenían crecimiento secundario (madera verdadera), desarrollaban miles de pequeñas raíces que crecían apretadas alrededor del tallo central para darle soporte y estabilidad.</t>
+  </si>
+  <si>
+    <t>Acadoparadoxides briareus</t>
+  </si>
+  <si>
+    <t>Formación Jbel Wawrmast, Alnif</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Minas de fosfato de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>. Conservado en matriz calcárea, con ligera alteración ferruginosa superficial. Este grupo de ammonites fue abundante en mares poco profundos del Jurásico medio y constituye un importante fósil guía para este intervalo.</t>
-    </r>
-  </si>
-  <si>
-    <t>Ammonite del Cretácico inferior con concha planiespiral evoluta. El pulido revela la compleja red de suturas internas, correspondientes a los tabiques que separaban las cámaras de flotación. Estas estructuras permitían al animal regular su posición en la columna de agua.</t>
-  </si>
-  <si>
-    <t>Ammonite caracterizado por una concha de enrollamiento evoluto y una ornamentación robusta de costillas radiales simples. El ejemplar presenta una preservación en matriz margo-caliza con una notable mineralización en limonita, responsable de su coloración ferruginosa. La matriz incluye restos fragmentarios de bivalvos (Ostreida), evidenciando un antiguo ecosistema de plataforma marina somera.</t>
-  </si>
-  <si>
-    <t>F-023</t>
-  </si>
-  <si>
-    <r>
-      <t>Lopha</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> sp.</t>
-    </r>
-  </si>
-  <si>
-    <t>Marruecos (Probable región del Atlas/Erfoud)</t>
-  </si>
-  <si>
-    <t>Bivalvia</t>
-  </si>
-  <si>
-    <t>Ostreida</t>
-  </si>
-  <si>
-    <t>Molusco Bivalvo</t>
-  </si>
-  <si>
-    <t>Molusco bivalvo inequivalve caracterizado por una fuerte ornamentación de costillas radiales ramificadas. Presenta una comisura marginal en zigzag (forma de "cresta de gallo") altamente pronunciada. Pieza de excepcional interés por su silicificación. El material biogénico original ha sido sustituido por sílice (calcedonia/microcuarzo), visible en el interior de las valvas por su textura vítrea y fractura concoidea. La matriz residual externa presenta tonalidades ocre típicas de sedimentos calcáreos meteorizados en climas áridos.</t>
-  </si>
-  <si>
-    <t>226 gr</t>
-  </si>
-  <si>
-    <t>7,3x8,1 cm</t>
-  </si>
-  <si>
-    <t>160 - 175 millones de años</t>
-  </si>
-  <si>
-    <t>145 - 160 millones de años</t>
-  </si>
-  <si>
-    <t>66 - 100 millones de años</t>
-  </si>
-  <si>
-    <t>100-145 millones de años</t>
-  </si>
-  <si>
-    <t>300 - 307 millones de años</t>
-  </si>
-  <si>
-    <t>235 - 250 millones de años</t>
-  </si>
-  <si>
-    <t>35- 55 millones de años</t>
+      <t>Khouribga</t>
+    </r>
+  </si>
+  <si>
+    <t>Rhacolepis sp.</t>
+  </si>
+  <si>
+    <t>90 - 100 millones de años</t>
+  </si>
+  <si>
+    <t>35 - 55 millones de años</t>
+  </si>
+  <si>
+    <t>100 - 145 millones de años</t>
+  </si>
+  <si>
+    <t>145  - 160 millones de años</t>
+  </si>
+  <si>
+    <t>485 – 500 millones de años</t>
+  </si>
+  <si>
+    <t>460 - 470 millones de años</t>
+  </si>
+  <si>
+    <t>Jurásico inferior</t>
+  </si>
+  <si>
+    <t>175 - 183 millones de años</t>
   </si>
 </sst>
 </file>
@@ -1541,13 +1544,13 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1556,16 +1559,16 @@
         <v>1</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1586,36 +1589,36 @@
         <v>8</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>171</v>
+        <v>225</v>
       </c>
       <c r="D2" t="s">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="F2" t="s">
-        <v>176</v>
+        <v>233</v>
       </c>
       <c r="G2" t="s">
-        <v>172</v>
+        <v>226</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
@@ -1627,325 +1630,325 @@
         <v>12</v>
       </c>
       <c r="K2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L2" t="s">
         <v>13</v>
       </c>
       <c r="N2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="P2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="F3" t="s">
+        <v>167</v>
+      </c>
+      <c r="G3" t="s">
         <v>174</v>
-      </c>
-      <c r="G3" t="s">
-        <v>186</v>
       </c>
       <c r="H3" t="s">
         <v>10</v>
       </c>
       <c r="I3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="K3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L3" t="s">
         <v>13</v>
       </c>
       <c r="N3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="O3" t="s">
+        <v>77</v>
+      </c>
+      <c r="P3" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q3" t="s">
         <v>79</v>
       </c>
-      <c r="P3" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>81</v>
-      </c>
       <c r="R3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="F4" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="G4" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="H4" t="s">
         <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="J4" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="K4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L4" t="s">
         <v>13</v>
       </c>
       <c r="N4" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="O4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="P4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Q4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C5" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="F5" t="s">
+        <v>167</v>
+      </c>
+      <c r="G5" t="s">
         <v>174</v>
-      </c>
-      <c r="G5" t="s">
-        <v>182</v>
       </c>
       <c r="H5" t="s">
         <v>10</v>
       </c>
       <c r="I5" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="J5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="K5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L5" t="s">
         <v>13</v>
       </c>
       <c r="N5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="O5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="P5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Q5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="D6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E6" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="F6" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="G6" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="H6" t="s">
         <v>10</v>
       </c>
       <c r="I6" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="K6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L6" t="s">
         <v>13</v>
       </c>
       <c r="N6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="O6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="P6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C7" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="D7" t="s">
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="F7" t="s">
-        <v>174</v>
+        <v>234</v>
       </c>
       <c r="G7" t="s">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="H7" t="s">
         <v>10</v>
       </c>
       <c r="I7" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="J7" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="K7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L7" t="s">
         <v>13</v>
       </c>
       <c r="N7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="O7" t="s">
-        <v>87</v>
+        <v>212</v>
       </c>
       <c r="P7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="R7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D8" t="s">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>85</v>
+        <v>181</v>
       </c>
       <c r="F8" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
       <c r="G8" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="H8" t="s">
         <v>10</v>
       </c>
       <c r="I8" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="J8" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="K8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L8" t="s">
         <v>16</v>
@@ -1954,54 +1957,54 @@
         <v>17</v>
       </c>
       <c r="N8" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O8" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D9" t="s">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>85</v>
+        <v>181</v>
       </c>
       <c r="F9" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
       <c r="G9" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="H9" t="s">
         <v>10</v>
       </c>
       <c r="I9" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="J9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="K9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L9" t="s">
         <v>16</v>
@@ -2010,54 +2013,54 @@
         <v>17</v>
       </c>
       <c r="N9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O9" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="P9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D10" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E10" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F10" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G10" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="H10" t="s">
         <v>10</v>
       </c>
       <c r="I10" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="J10" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="K10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L10" t="s">
         <v>16</v>
@@ -2066,54 +2069,54 @@
         <v>17</v>
       </c>
       <c r="N10" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="P10" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Q10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R10" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E11" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F11" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G11" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="H11" t="s">
         <v>10</v>
       </c>
       <c r="I11" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J11" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="K11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L11" t="s">
         <v>16</v>
@@ -2122,54 +2125,54 @@
         <v>17</v>
       </c>
       <c r="N11" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="P11" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="Q11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R11" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G12" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="H12" t="s">
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="J12" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="K12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L12" t="s">
         <v>16</v>
@@ -2178,54 +2181,54 @@
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O12" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="P12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R12" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F13" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G13" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="H13" t="s">
         <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="J13" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="K13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L13" t="s">
         <v>16</v>
@@ -2234,39 +2237,39 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O13" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="P13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R13" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C14" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D14" t="s">
         <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>188</v>
+        <v>235</v>
       </c>
       <c r="F14" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
@@ -2275,13 +2278,13 @@
         <v>20</v>
       </c>
       <c r="I14" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="J14" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="K14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L14" t="s">
         <v>16</v>
@@ -2293,51 +2296,51 @@
         <v>24</v>
       </c>
       <c r="O14" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="P14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C15" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="D15" t="s">
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="F15" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="G15" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="H15" t="s">
         <v>22</v>
       </c>
       <c r="I15" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="J15" t="s">
         <v>23</v>
       </c>
       <c r="K15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L15" t="s">
         <v>16</v>
@@ -2349,51 +2352,51 @@
         <v>24</v>
       </c>
       <c r="O15" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="P15" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q15" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C16" t="s">
-        <v>156</v>
+        <v>216</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E16" t="s">
-        <v>102</v>
+        <v>166</v>
       </c>
       <c r="F16" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="G16" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="H16" t="s">
         <v>10</v>
       </c>
       <c r="I16" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="J16" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="K16" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L16" t="s">
         <v>16</v>
@@ -2405,51 +2408,51 @@
         <v>24</v>
       </c>
       <c r="O16" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="P16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q16" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R16" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C17" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E17" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F17" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="G17" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="H17" t="s">
         <v>10</v>
       </c>
       <c r="I17" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="J17" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="K17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L17" t="s">
         <v>16</v>
@@ -2461,51 +2464,51 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="P17" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R17" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>213</v>
       </c>
       <c r="C18" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="E18" t="s">
-        <v>103</v>
+        <v>183</v>
       </c>
       <c r="F18" t="s">
-        <v>228</v>
+        <v>177</v>
       </c>
       <c r="G18" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
       <c r="H18" t="s">
-        <v>197</v>
+        <v>10</v>
       </c>
       <c r="I18" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="J18" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="K18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L18" t="s">
         <v>16</v>
@@ -2514,39 +2517,39 @@
         <v>21</v>
       </c>
       <c r="N18" t="s">
-        <v>24</v>
+        <v>214</v>
       </c>
       <c r="O18" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="P18" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q18" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R18" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F19" t="s">
-        <v>229</v>
+        <v>208</v>
       </c>
       <c r="G19" t="s">
         <v>26</v>
@@ -2555,54 +2558,54 @@
         <v>27</v>
       </c>
       <c r="I19" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="J19" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="K19" t="s">
         <v>28</v>
       </c>
       <c r="L19" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="M19" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="N19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O19" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="P19" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R19" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" t="s">
+        <v>109</v>
+      </c>
+      <c r="E20" t="s">
         <v>110</v>
       </c>
-      <c r="C20" t="s">
-        <v>109</v>
-      </c>
-      <c r="D20" t="s">
-        <v>112</v>
-      </c>
-      <c r="E20" t="s">
-        <v>113</v>
-      </c>
       <c r="F20" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -2611,255 +2614,255 @@
         <v>31</v>
       </c>
       <c r="I20" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="J20" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="K20" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L20" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="M20" t="s">
+        <v>105</v>
+      </c>
+      <c r="N20" t="s">
+        <v>88</v>
+      </c>
+      <c r="O20" t="s">
         <v>108</v>
       </c>
-      <c r="N20" t="s">
-        <v>91</v>
-      </c>
-      <c r="O20" t="s">
+      <c r="P20" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q20" t="s">
         <v>111</v>
       </c>
-      <c r="P20" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>114</v>
-      </c>
       <c r="R20" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C21" t="s">
         <v>32</v>
       </c>
       <c r="D21" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="E21" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="F21" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="G21" t="s">
+        <v>223</v>
+      </c>
+      <c r="H21" t="s">
         <v>33</v>
       </c>
-      <c r="H21" t="s">
-        <v>34</v>
-      </c>
       <c r="I21" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="J21" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K21" t="s">
         <v>28</v>
       </c>
       <c r="L21" t="s">
+        <v>112</v>
+      </c>
+      <c r="M21" t="s">
         <v>115</v>
       </c>
-      <c r="M21" t="s">
-        <v>119</v>
-      </c>
       <c r="N21" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="O21" t="s">
-        <v>117</v>
+        <v>224</v>
       </c>
       <c r="P21" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="Q21" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R21" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B22" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C22" t="s">
+        <v>228</v>
+      </c>
+      <c r="D22" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" t="s">
+        <v>100</v>
+      </c>
+      <c r="F22" t="s">
+        <v>231</v>
+      </c>
+      <c r="G22" t="s">
+        <v>194</v>
+      </c>
+      <c r="H22" t="s">
+        <v>33</v>
+      </c>
+      <c r="I22" t="s">
+        <v>164</v>
+      </c>
+      <c r="J22" t="s">
+        <v>162</v>
+      </c>
+      <c r="K22" t="s">
         <v>36</v>
       </c>
-      <c r="D22" t="s">
+      <c r="L22" t="s">
         <v>37</v>
       </c>
-      <c r="E22" t="s">
-        <v>103</v>
-      </c>
-      <c r="F22" t="s">
-        <v>228</v>
-      </c>
-      <c r="G22" t="s">
-        <v>208</v>
-      </c>
-      <c r="H22" t="s">
-        <v>34</v>
-      </c>
-      <c r="I22" t="s">
-        <v>169</v>
-      </c>
-      <c r="J22" t="s">
-        <v>167</v>
-      </c>
-      <c r="K22" t="s">
+      <c r="M22" t="s">
         <v>38</v>
       </c>
-      <c r="L22" t="s">
-        <v>39</v>
-      </c>
-      <c r="M22" t="s">
-        <v>40</v>
-      </c>
       <c r="N22" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="O22" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="P22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R22" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C23" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="F23" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G23" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="H23" t="s">
         <v>10</v>
       </c>
       <c r="I23" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="J23" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="K23" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="L23" t="s">
+        <v>39</v>
+      </c>
+      <c r="M23" t="s">
+        <v>40</v>
+      </c>
+      <c r="N23" t="s">
         <v>41</v>
       </c>
-      <c r="M23" t="s">
-        <v>42</v>
-      </c>
-      <c r="N23" t="s">
-        <v>43</v>
-      </c>
       <c r="O23" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="P23" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q23" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R23" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="B24" t="s">
-        <v>221</v>
+        <v>204</v>
       </c>
       <c r="C24" t="s">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="D24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E24" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F24" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G24" t="s">
-        <v>218</v>
+        <v>201</v>
       </c>
       <c r="H24" t="s">
         <v>10</v>
       </c>
       <c r="I24" t="s">
-        <v>224</v>
+        <v>207</v>
       </c>
       <c r="J24" t="s">
-        <v>223</v>
+        <v>206</v>
       </c>
       <c r="K24" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L24" t="s">
-        <v>219</v>
+        <v>202</v>
       </c>
       <c r="N24" t="s">
-        <v>220</v>
+        <v>203</v>
       </c>
       <c r="O24" t="s">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="P24" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Q24" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="R24" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización piece F-003: Procedencia y País
</commit_message>
<xml_diff>
--- a/Coleccion de Fosiles.xlsx
+++ b/Coleccion de Fosiles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coleccion Fósiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E11956B-ADFE-440D-A043-047FE0AE2DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6235E247-8836-4C78-893E-02F81050A532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="236">
   <si>
     <t>Periodo</t>
   </si>
@@ -826,9 +826,6 @@
   </si>
   <si>
     <t>Illaenus sp.</t>
-  </si>
-  <si>
-    <t>Yacimientos del río Volkhov (probable)</t>
   </si>
   <si>
     <t>Género</t>
@@ -1550,7 +1547,7 @@
         <v>70</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1606,19 +1603,19 @@
         <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D2" t="s">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
@@ -1665,13 +1662,13 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F3" t="s">
         <v>167</v>
       </c>
       <c r="G3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H3" t="s">
         <v>10</v>
@@ -1718,16 +1715,16 @@
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="H4" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="I4" t="s">
         <v>133</v>
@@ -1765,19 +1762,19 @@
         <v>76</v>
       </c>
       <c r="C5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F5" t="s">
         <v>167</v>
       </c>
       <c r="G5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H5" t="s">
         <v>10</v>
@@ -1818,19 +1815,19 @@
         <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D6" t="s">
         <v>83</v>
       </c>
       <c r="E6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F6" t="s">
+        <v>176</v>
+      </c>
+      <c r="G6" t="s">
         <v>177</v>
-      </c>
-      <c r="G6" t="s">
-        <v>178</v>
       </c>
       <c r="H6" t="s">
         <v>10</v>
@@ -1871,19 +1868,19 @@
         <v>76</v>
       </c>
       <c r="C7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D7" t="s">
         <v>14</v>
       </c>
       <c r="E7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F7" t="s">
+        <v>233</v>
+      </c>
+      <c r="G7" t="s">
         <v>210</v>
-      </c>
-      <c r="F7" t="s">
-        <v>234</v>
-      </c>
-      <c r="G7" t="s">
-        <v>211</v>
       </c>
       <c r="H7" t="s">
         <v>10</v>
@@ -1904,7 +1901,7 @@
         <v>68</v>
       </c>
       <c r="O7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="P7" t="s">
         <v>80</v>
@@ -1924,19 +1921,19 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D8" t="s">
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F8" t="s">
         <v>167</v>
       </c>
       <c r="G8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H8" t="s">
         <v>10</v>
@@ -1980,19 +1977,19 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D9" t="s">
         <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F9" t="s">
         <v>167</v>
       </c>
       <c r="G9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H9" t="s">
         <v>10</v>
@@ -2036,7 +2033,7 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D10" t="s">
         <v>83</v>
@@ -2045,10 +2042,10 @@
         <v>83</v>
       </c>
       <c r="F10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H10" t="s">
         <v>10</v>
@@ -2092,7 +2089,7 @@
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D11" t="s">
         <v>83</v>
@@ -2101,10 +2098,10 @@
         <v>83</v>
       </c>
       <c r="F11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H11" t="s">
         <v>10</v>
@@ -2148,7 +2145,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D12" t="s">
         <v>83</v>
@@ -2157,10 +2154,10 @@
         <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H12" t="s">
         <v>10</v>
@@ -2204,7 +2201,7 @@
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D13" t="s">
         <v>83</v>
@@ -2213,10 +2210,10 @@
         <v>83</v>
       </c>
       <c r="F13" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H13" t="s">
         <v>10</v>
@@ -2266,10 +2263,10 @@
         <v>18</v>
       </c>
       <c r="E14" t="s">
+        <v>234</v>
+      </c>
+      <c r="F14" t="s">
         <v>235</v>
-      </c>
-      <c r="F14" t="s">
-        <v>236</v>
       </c>
       <c r="G14" t="s">
         <v>19</v>
@@ -2296,7 +2293,7 @@
         <v>24</v>
       </c>
       <c r="O14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="P14" t="s">
         <v>80</v>
@@ -2316,7 +2313,7 @@
         <v>96</v>
       </c>
       <c r="C15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D15" t="s">
         <v>18</v>
@@ -2325,7 +2322,7 @@
         <v>166</v>
       </c>
       <c r="F15" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G15" t="s">
         <v>98</v>
@@ -2372,7 +2369,7 @@
         <v>96</v>
       </c>
       <c r="C16" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D16" t="s">
         <v>18</v>
@@ -2381,10 +2378,10 @@
         <v>166</v>
       </c>
       <c r="F16" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H16" t="s">
         <v>10</v>
@@ -2408,7 +2405,7 @@
         <v>24</v>
       </c>
       <c r="O16" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="P16" t="s">
         <v>80</v>
@@ -2428,7 +2425,7 @@
         <v>96</v>
       </c>
       <c r="C17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D17" t="s">
         <v>35</v>
@@ -2437,10 +2434,10 @@
         <v>100</v>
       </c>
       <c r="F17" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H17" t="s">
         <v>10</v>
@@ -2464,7 +2461,7 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="P17" t="s">
         <v>80</v>
@@ -2481,22 +2478,22 @@
         <v>59</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C18" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D18" t="s">
         <v>83</v>
       </c>
       <c r="E18" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F18" t="s">
+        <v>176</v>
+      </c>
+      <c r="G18" t="s">
         <v>177</v>
-      </c>
-      <c r="G18" t="s">
-        <v>178</v>
       </c>
       <c r="H18" t="s">
         <v>10</v>
@@ -2517,10 +2514,10 @@
         <v>21</v>
       </c>
       <c r="N18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="O18" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="P18" t="s">
         <v>80</v>
@@ -2540,7 +2537,7 @@
         <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
@@ -2549,7 +2546,7 @@
         <v>102</v>
       </c>
       <c r="F19" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G19" t="s">
         <v>26</v>
@@ -2567,10 +2564,10 @@
         <v>28</v>
       </c>
       <c r="L19" t="s">
+        <v>186</v>
+      </c>
+      <c r="M19" t="s">
         <v>187</v>
-      </c>
-      <c r="M19" t="s">
-        <v>188</v>
       </c>
       <c r="N19" t="s">
         <v>34</v>
@@ -2605,7 +2602,7 @@
         <v>110</v>
       </c>
       <c r="F20" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -2655,16 +2652,16 @@
         <v>32</v>
       </c>
       <c r="D21" t="s">
+        <v>219</v>
+      </c>
+      <c r="E21" t="s">
         <v>220</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>221</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>222</v>
-      </c>
-      <c r="G21" t="s">
-        <v>223</v>
       </c>
       <c r="H21" t="s">
         <v>33</v>
@@ -2688,7 +2685,7 @@
         <v>116</v>
       </c>
       <c r="O21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="P21" t="s">
         <v>114</v>
@@ -2708,7 +2705,7 @@
         <v>118</v>
       </c>
       <c r="C22" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D22" t="s">
         <v>35</v>
@@ -2717,10 +2714,10 @@
         <v>100</v>
       </c>
       <c r="F22" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G22" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H22" t="s">
         <v>33</v>
@@ -2741,7 +2738,7 @@
         <v>38</v>
       </c>
       <c r="N22" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O22" t="s">
         <v>117</v>
@@ -2764,19 +2761,19 @@
         <v>119</v>
       </c>
       <c r="C23" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G23" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H23" t="s">
         <v>10</v>
@@ -2814,13 +2811,13 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>198</v>
+      </c>
+      <c r="B24" t="s">
+        <v>203</v>
+      </c>
+      <c r="C24" t="s">
         <v>199</v>
-      </c>
-      <c r="B24" t="s">
-        <v>204</v>
-      </c>
-      <c r="C24" t="s">
-        <v>200</v>
       </c>
       <c r="D24" t="s">
         <v>35</v>
@@ -2829,31 +2826,31 @@
         <v>99</v>
       </c>
       <c r="F24" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G24" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H24" t="s">
         <v>10</v>
       </c>
       <c r="I24" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J24" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K24" t="s">
         <v>88</v>
       </c>
       <c r="L24" t="s">
+        <v>201</v>
+      </c>
+      <c r="N24" t="s">
         <v>202</v>
       </c>
-      <c r="N24" t="s">
-        <v>203</v>
-      </c>
       <c r="O24" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P24" t="s">
         <v>78</v>

</xml_diff>